<commit_message>
Bug fixed- Empty observer table looks well now
</commit_message>
<xml_diff>
--- a/src/main/resources/documents/2026/prijedlozi BO/03548  Koalicija za državu Birački odbori.xlsx
+++ b/src/main/resources/documents/2026/prijedlozi BO/03548  Koalicija za državu Birački odbori.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vladanmalinic/Documents/GitHub/flow-crm-tutorial/src/main/resources/documents/2026/prijedlozi BO/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A486F16-424C-FF45-84DA-D3DA5FD9BCDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDDE4EA4-C243-B042-B2D1-C7287E6FAF63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -100,6 +100,9 @@
     <t>АДА - 4, ПШ "ВУК С. КАРАЏИЋ", Вељка Млађеновића бб, уч. 4</t>
   </si>
   <si>
+    <t>Анастасија Двизац</t>
+  </si>
+  <si>
     <t>ВСС-инжињер рачунарства</t>
   </si>
   <si>
@@ -148,6 +151,9 @@
     <t>БОРИК I /5, ОШ "ВУК С. КАРАЏИЋ", Саве Ковачевића бб, уч. 5</t>
   </si>
   <si>
+    <t>Немања Паламета</t>
+  </si>
+  <si>
     <t>ССС-угоститељ</t>
   </si>
   <si>
@@ -373,6 +379,9 @@
     <t>ДРАГОЧАЈ – 1, ОШ "ДЕСАНКА МАКСИМОВИЋ", Драгочај, уч. 2</t>
   </si>
   <si>
+    <t>Ана Хајдер</t>
+  </si>
+  <si>
     <t>ССС-медицински техничар</t>
   </si>
   <si>
@@ -460,6 +469,9 @@
     <t>КОЛА - 1, ОШ "ПЕТАР КОЧИЋ", Кола, уч. 1</t>
   </si>
   <si>
+    <t>Кларета Кречар</t>
+  </si>
+  <si>
     <t>ССС-лаборант</t>
   </si>
   <si>
@@ -472,6 +484,9 @@
     <t>5550078104677535</t>
   </si>
   <si>
+    <t>Жељко Кречар</t>
+  </si>
+  <si>
     <t>ССС-техничар</t>
   </si>
   <si>
@@ -490,6 +505,9 @@
     <t>КОЧИЋЕВ ВИЈЕНАЦ - 4, ОШ "ЗМАЈ Ј. ЈОВАНОВИЋ", Бранка Загорца 1, уч. 4</t>
   </si>
   <si>
+    <t>Амела Курјак</t>
+  </si>
+  <si>
     <t>ВСС-просветни радник</t>
   </si>
   <si>
@@ -502,6 +520,9 @@
     <t>5621008018366541</t>
   </si>
   <si>
+    <t>Адмира Курјак</t>
+  </si>
+  <si>
     <t>0208983105068</t>
   </si>
   <si>
@@ -547,6 +568,9 @@
     <t>ЛАЗАРЕВО I / 2, ПОЉОПОРИВРЕДНА ШКОЛА, Књаза Милоша 9, уч. 2</t>
   </si>
   <si>
+    <t>Младен Ћук</t>
+  </si>
+  <si>
     <t>0301003152723</t>
   </si>
   <si>
@@ -562,6 +586,9 @@
     <t>ЛАЗАРЕВО I / 6, ОШ "БОРИСАВ СТАНКОВИЋ", Ивана Косанчића 2, уч. 2</t>
   </si>
   <si>
+    <t>Вук Шмуља</t>
+  </si>
+  <si>
     <t>ССС-гимназија</t>
   </si>
   <si>
@@ -784,6 +811,9 @@
     <t>ОБИЛИЋЕВО I / 9, ОШ "ПЕТАР П. ЊЕГОШ", Бул. В. С. Степановића 28, уч. 9</t>
   </si>
   <si>
+    <t>Давор Папоња</t>
+  </si>
+  <si>
     <t>ВСС-наставник ликовне кул.</t>
   </si>
   <si>
@@ -802,6 +832,9 @@
     <t>ОБИЛИЋЕВО II / 2, ОШ "ДОСИТЕЈ ОБРАДОВИЋ", Мирка Ковачевића 27, уч. 2</t>
   </si>
   <si>
+    <t>Маја Келеч</t>
+  </si>
+  <si>
     <t>ВСС-дипл.економиста</t>
   </si>
   <si>
@@ -895,6 +928,9 @@
     <t>ПАПРИКОВАЦ 3, ШКОЛА ЗА СЛУШНО ОШТЕЋЕНЕ, Др Ј. Рашковића 28, уч. 3</t>
   </si>
   <si>
+    <t>Вања Праштало</t>
+  </si>
+  <si>
     <t>ССС-стоматолошки техничар</t>
   </si>
   <si>
@@ -1123,6 +1159,9 @@
     <t>СТАРЧЕВИЦА 5, ОШ "БРАНКО РАДИЧЕВИЋ", Булев. В. С. Степановића 116, уч. 4</t>
   </si>
   <si>
+    <t>Лука Марјанац</t>
+  </si>
+  <si>
     <t>2102005100032</t>
   </si>
   <si>
@@ -1138,6 +1177,9 @@
     <t>СТАРЧЕВИЦА 9, ОШ "БРАНКО РАДИЧЕВИЋ", Булев. В. С. Степановића 116, уч. 8</t>
   </si>
   <si>
+    <t>Владимир Деспот</t>
+  </si>
+  <si>
     <t>ССС-саобраћајни техничар</t>
   </si>
   <si>
@@ -1174,6 +1216,9 @@
     <t>1613000094199083</t>
   </si>
   <si>
+    <t>Ненад Хајдер</t>
+  </si>
+  <si>
     <t>ВСС-дипл.инг.шумарства</t>
   </si>
   <si>
@@ -1288,6 +1333,9 @@
     <t>ЦЕНТАР II / 2, ОШ "ИВО АНДРИЋ", Бранка Радичевића 16, уч. 1</t>
   </si>
   <si>
+    <t>Миранда Берендика</t>
+  </si>
+  <si>
     <t>2305990188737</t>
   </si>
   <si>
@@ -1303,6 +1351,9 @@
     <t>ЦЕНТАР II / 6, ОШ "ИВО АНДРИЋ", Бранка Радичевића 16, уч. 5</t>
   </si>
   <si>
+    <t>Саша Берендика</t>
+  </si>
+  <si>
     <t>ВСС-дипл.журналиста</t>
   </si>
   <si>
@@ -1321,6 +1372,9 @@
     <t>ЧЕСМА 2, МЗ ЧЕСМА, Петра Великог 30, сала 1</t>
   </si>
   <si>
+    <t>Тамара Ољача</t>
+  </si>
+  <si>
     <t>ССС-хемијски тех.</t>
   </si>
   <si>
@@ -1444,6 +1498,9 @@
     <t>КАРАНОВАЦ - 3, ОШ "МИЛАН РАКИЋ", Карановац, уч. 3</t>
   </si>
   <si>
+    <t>Немања Копрена</t>
+  </si>
+  <si>
     <t>ССС-радник</t>
   </si>
   <si>
@@ -1460,63 +1517,6 @@
   </si>
   <si>
     <t>__________________________________________</t>
-  </si>
-  <si>
-    <t>Анастасија Двизац</t>
-  </si>
-  <si>
-    <t>Немања Паламета</t>
-  </si>
-  <si>
-    <t>Ана Хајдер</t>
-  </si>
-  <si>
-    <t>Кларета Кречар</t>
-  </si>
-  <si>
-    <t>Жељко Кречар</t>
-  </si>
-  <si>
-    <t>Адмира Курјак</t>
-  </si>
-  <si>
-    <t>Младен Ћук</t>
-  </si>
-  <si>
-    <t>Вук Шмуља</t>
-  </si>
-  <si>
-    <t>Давор Папоња</t>
-  </si>
-  <si>
-    <t>Маја Келеч</t>
-  </si>
-  <si>
-    <t>Вања Праштало</t>
-  </si>
-  <si>
-    <t>Лука Марјанац</t>
-  </si>
-  <si>
-    <t>Владимир Деспот</t>
-  </si>
-  <si>
-    <t>Ненад Хајдер</t>
-  </si>
-  <si>
-    <t>Миранда Берендика</t>
-  </si>
-  <si>
-    <t>Саша Берендика</t>
-  </si>
-  <si>
-    <t>Тамара Ољача</t>
-  </si>
-  <si>
-    <t>Немања Копрена</t>
-  </si>
-  <si>
-    <t>Амела Курјак</t>
   </si>
 </sst>
 </file>
@@ -1801,15 +1801,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Excel Built-in Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
@@ -2150,13 +2150,13 @@
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="26" t="s">
+      <c r="D2" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="28"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="26"/>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
       <c r="K2" s="3"/>
@@ -2245,13 +2245,13 @@
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="26" t="s">
+      <c r="D7" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="27"/>
-      <c r="F7" s="27"/>
-      <c r="G7" s="27"/>
-      <c r="H7" s="28"/>
+      <c r="E7" s="25"/>
+      <c r="F7" s="25"/>
+      <c r="G7" s="25"/>
+      <c r="H7" s="26"/>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
       <c r="K7" s="3"/>
@@ -2281,25 +2281,25 @@
       </c>
       <c r="B9" s="5"/>
       <c r="D9" t="s">
-        <v>480</v>
+        <v>26</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="J9" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K9" s="5"/>
       <c r="L9" s="5"/>
@@ -2336,17 +2336,17 @@
     </row>
     <row r="12" spans="1:12" ht="15.5" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
-      <c r="D12" s="26" t="s">
-        <v>33</v>
-      </c>
-      <c r="E12" s="27"/>
-      <c r="F12" s="27"/>
-      <c r="G12" s="27"/>
-      <c r="H12" s="28"/>
+      <c r="D12" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="E12" s="25"/>
+      <c r="F12" s="25"/>
+      <c r="G12" s="25"/>
+      <c r="H12" s="26"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
       <c r="K12" s="3"/>
@@ -2376,25 +2376,25 @@
       </c>
       <c r="B14" s="5"/>
       <c r="D14" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="J14" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K14" s="5"/>
       <c r="L14" s="5"/>
@@ -2431,17 +2431,17 @@
     </row>
     <row r="17" spans="1:12" ht="15.5" customHeight="1">
       <c r="A17" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
-      <c r="D17" s="26" t="s">
-        <v>41</v>
-      </c>
-      <c r="E17" s="27"/>
-      <c r="F17" s="27"/>
-      <c r="G17" s="27"/>
-      <c r="H17" s="28"/>
+      <c r="D17" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="E17" s="25"/>
+      <c r="F17" s="25"/>
+      <c r="G17" s="25"/>
+      <c r="H17" s="26"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
       <c r="K17" s="3"/>
@@ -2471,19 +2471,19 @@
       </c>
       <c r="B19" s="5"/>
       <c r="D19" t="s">
-        <v>481</v>
+        <v>43</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F19" s="6" t="s">
         <v>18</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I19" s="5"/>
       <c r="J19" s="4"/>
@@ -2522,17 +2522,17 @@
     </row>
     <row r="22" spans="1:12" ht="15.5" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
-      <c r="D22" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="E22" s="27"/>
-      <c r="F22" s="27"/>
-      <c r="G22" s="27"/>
-      <c r="H22" s="28"/>
+      <c r="D22" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="E22" s="25"/>
+      <c r="F22" s="25"/>
+      <c r="G22" s="25"/>
+      <c r="H22" s="26"/>
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
       <c r="K22" s="3"/>
@@ -2562,22 +2562,22 @@
       </c>
       <c r="B24" s="5"/>
       <c r="D24" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="I24" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="J24" s="7" t="s">
         <v>22</v>
@@ -2617,17 +2617,17 @@
     </row>
     <row r="27" spans="1:12" ht="15.5" customHeight="1">
       <c r="A27" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
-      <c r="D27" s="26" t="s">
-        <v>54</v>
-      </c>
-      <c r="E27" s="27"/>
-      <c r="F27" s="27"/>
-      <c r="G27" s="27"/>
-      <c r="H27" s="28"/>
+      <c r="D27" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="E27" s="25"/>
+      <c r="F27" s="25"/>
+      <c r="G27" s="25"/>
+      <c r="H27" s="26"/>
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
       <c r="K27" s="3"/>
@@ -2657,25 +2657,25 @@
       </c>
       <c r="B29" s="5"/>
       <c r="D29" s="8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F29" s="6" t="s">
         <v>18</v>
       </c>
       <c r="G29" s="6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I29" s="6" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="J29" s="7" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="K29" s="5"/>
       <c r="L29" s="5"/>
@@ -2712,17 +2712,17 @@
     </row>
     <row r="32" spans="1:12" ht="15.5" customHeight="1">
       <c r="A32" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
-      <c r="D32" s="26" t="s">
-        <v>62</v>
-      </c>
-      <c r="E32" s="27"/>
-      <c r="F32" s="27"/>
-      <c r="G32" s="27"/>
-      <c r="H32" s="28"/>
+      <c r="D32" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="E32" s="25"/>
+      <c r="F32" s="25"/>
+      <c r="G32" s="25"/>
+      <c r="H32" s="26"/>
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
       <c r="K32" s="3"/>
@@ -2752,7 +2752,7 @@
       </c>
       <c r="B34" s="5"/>
       <c r="D34" s="21" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E34" s="15" t="s">
         <v>17</v>
@@ -2761,16 +2761,16 @@
         <v>18</v>
       </c>
       <c r="G34" s="16" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H34" s="16" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I34" s="16" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="J34" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K34" s="5"/>
       <c r="L34" s="5"/>
@@ -2807,17 +2807,17 @@
     </row>
     <row r="37" spans="1:12" ht="15.5" customHeight="1">
       <c r="A37" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
-      <c r="D37" s="26" t="s">
-        <v>68</v>
-      </c>
-      <c r="E37" s="27"/>
-      <c r="F37" s="27"/>
-      <c r="G37" s="27"/>
-      <c r="H37" s="28"/>
+      <c r="D37" s="24" t="s">
+        <v>70</v>
+      </c>
+      <c r="E37" s="25"/>
+      <c r="F37" s="25"/>
+      <c r="G37" s="25"/>
+      <c r="H37" s="26"/>
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
       <c r="K37" s="3"/>
@@ -2847,25 +2847,25 @@
       </c>
       <c r="B39" s="5"/>
       <c r="D39" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E39" s="4" t="s">
         <v>17</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H39" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I39" s="5" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="J39" s="4" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="K39" s="5"/>
       <c r="L39" s="5"/>
@@ -2902,17 +2902,17 @@
     </row>
     <row r="42" spans="1:12" ht="15.5" customHeight="1">
       <c r="A42" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
-      <c r="D42" s="26" t="s">
-        <v>75</v>
-      </c>
-      <c r="E42" s="27"/>
-      <c r="F42" s="27"/>
-      <c r="G42" s="27"/>
-      <c r="H42" s="28"/>
+      <c r="D42" s="24" t="s">
+        <v>77</v>
+      </c>
+      <c r="E42" s="25"/>
+      <c r="F42" s="25"/>
+      <c r="G42" s="25"/>
+      <c r="H42" s="26"/>
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
       <c r="K42" s="3"/>
@@ -2942,25 +2942,25 @@
       </c>
       <c r="B44" s="5"/>
       <c r="D44" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E44" s="7" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F44" s="6" t="s">
         <v>18</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="I44" s="6" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="J44" s="7" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="K44" s="5"/>
       <c r="L44" s="5"/>
@@ -2997,17 +2997,17 @@
     </row>
     <row r="47" spans="1:12" ht="15.5" customHeight="1">
       <c r="A47" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
-      <c r="D47" s="26" t="s">
-        <v>83</v>
-      </c>
-      <c r="E47" s="27"/>
-      <c r="F47" s="27"/>
-      <c r="G47" s="27"/>
-      <c r="H47" s="28"/>
+      <c r="D47" s="24" t="s">
+        <v>85</v>
+      </c>
+      <c r="E47" s="25"/>
+      <c r="F47" s="25"/>
+      <c r="G47" s="25"/>
+      <c r="H47" s="26"/>
       <c r="I47" s="2"/>
       <c r="J47" s="2"/>
       <c r="K47" s="3"/>
@@ -3037,25 +3037,25 @@
       </c>
       <c r="B49" s="5"/>
       <c r="D49" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E49" s="7" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F49" s="6" t="s">
         <v>18</v>
       </c>
       <c r="G49" s="6" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="I49" s="6" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="J49" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K49" s="5"/>
       <c r="L49" s="5"/>
@@ -3092,17 +3092,17 @@
     </row>
     <row r="52" spans="1:12" ht="15.5" customHeight="1">
       <c r="A52" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
-      <c r="D52" s="26" t="s">
-        <v>90</v>
-      </c>
-      <c r="E52" s="27"/>
-      <c r="F52" s="27"/>
-      <c r="G52" s="27"/>
-      <c r="H52" s="28"/>
+      <c r="D52" s="24" t="s">
+        <v>92</v>
+      </c>
+      <c r="E52" s="25"/>
+      <c r="F52" s="25"/>
+      <c r="G52" s="25"/>
+      <c r="H52" s="26"/>
       <c r="I52" s="2"/>
       <c r="J52" s="2"/>
       <c r="K52" s="3"/>
@@ -3132,25 +3132,25 @@
       </c>
       <c r="B54" s="5"/>
       <c r="D54" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E54" s="7" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F54" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G54" s="6" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="H54" s="22" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="I54" s="6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J54" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="K54" s="5"/>
       <c r="L54" s="5"/>
@@ -3187,17 +3187,17 @@
     </row>
     <row r="57" spans="1:12" ht="15.5" customHeight="1">
       <c r="A57" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B57" s="2"/>
       <c r="C57" s="2"/>
-      <c r="D57" s="26" t="s">
-        <v>98</v>
-      </c>
-      <c r="E57" s="27"/>
-      <c r="F57" s="27"/>
-      <c r="G57" s="27"/>
-      <c r="H57" s="28"/>
+      <c r="D57" s="24" t="s">
+        <v>100</v>
+      </c>
+      <c r="E57" s="25"/>
+      <c r="F57" s="25"/>
+      <c r="G57" s="25"/>
+      <c r="H57" s="26"/>
       <c r="I57" s="2"/>
       <c r="J57" s="2"/>
       <c r="K57" s="3"/>
@@ -3227,25 +3227,25 @@
       </c>
       <c r="B59" s="5"/>
       <c r="D59" s="21" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E59" s="15" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="F59" s="16" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="16" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H59" s="16" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="I59" s="16" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="J59" s="15" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="K59" s="5"/>
       <c r="L59" s="5"/>
@@ -3282,17 +3282,17 @@
     </row>
     <row r="62" spans="1:12" ht="15.5" customHeight="1">
       <c r="A62" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B62" s="2"/>
       <c r="C62" s="2"/>
-      <c r="D62" s="26" t="s">
-        <v>106</v>
-      </c>
-      <c r="E62" s="27"/>
-      <c r="F62" s="27"/>
-      <c r="G62" s="27"/>
-      <c r="H62" s="28"/>
+      <c r="D62" s="24" t="s">
+        <v>108</v>
+      </c>
+      <c r="E62" s="25"/>
+      <c r="F62" s="25"/>
+      <c r="G62" s="25"/>
+      <c r="H62" s="26"/>
       <c r="I62" s="2"/>
       <c r="J62" s="2"/>
       <c r="K62" s="3"/>
@@ -3322,7 +3322,7 @@
       </c>
       <c r="B64" s="5"/>
       <c r="D64" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E64" t="s">
         <v>17</v>
@@ -3334,13 +3334,13 @@
         <v>2209974100030</v>
       </c>
       <c r="H64" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I64" s="18">
         <v>1545049939838570</v>
       </c>
       <c r="J64" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="K64" s="5"/>
       <c r="L64" s="5"/>
@@ -3367,42 +3367,42 @@
       </c>
       <c r="B66" s="5"/>
       <c r="D66" s="21" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E66" s="15" t="s">
         <v>17</v>
       </c>
       <c r="F66" s="16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G66" s="16" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H66" s="16" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="I66" s="16" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="J66" s="15" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="K66" s="5"/>
       <c r="L66" s="5"/>
     </row>
     <row r="67" spans="1:12" ht="15.5" customHeight="1">
       <c r="A67" s="2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B67" s="2"/>
       <c r="C67" s="2"/>
-      <c r="D67" s="26" t="s">
-        <v>116</v>
-      </c>
-      <c r="E67" s="27"/>
-      <c r="F67" s="27"/>
-      <c r="G67" s="27"/>
-      <c r="H67" s="28"/>
+      <c r="D67" s="24" t="s">
+        <v>118</v>
+      </c>
+      <c r="E67" s="25"/>
+      <c r="F67" s="25"/>
+      <c r="G67" s="25"/>
+      <c r="H67" s="26"/>
       <c r="I67" s="2"/>
       <c r="J67" s="2"/>
       <c r="K67" s="3"/>
@@ -3432,25 +3432,25 @@
       </c>
       <c r="B69" s="5"/>
       <c r="D69" t="s">
-        <v>482</v>
+        <v>119</v>
       </c>
       <c r="E69" s="7" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="F69" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G69" s="6" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="H69" s="6" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="I69" s="6" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="J69" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K69" s="5"/>
       <c r="L69" s="5"/>
@@ -3487,17 +3487,17 @@
     </row>
     <row r="72" spans="1:12" ht="15.5" customHeight="1">
       <c r="A72" s="2" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B72" s="2"/>
       <c r="C72" s="2"/>
-      <c r="D72" s="26" t="s">
-        <v>122</v>
-      </c>
-      <c r="E72" s="27"/>
-      <c r="F72" s="27"/>
-      <c r="G72" s="27"/>
-      <c r="H72" s="28"/>
+      <c r="D72" s="24" t="s">
+        <v>125</v>
+      </c>
+      <c r="E72" s="25"/>
+      <c r="F72" s="25"/>
+      <c r="G72" s="25"/>
+      <c r="H72" s="26"/>
       <c r="I72" s="2"/>
       <c r="J72" s="2"/>
       <c r="K72" s="3"/>
@@ -3527,25 +3527,25 @@
       </c>
       <c r="B74" s="5"/>
       <c r="D74" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E74" s="7" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F74" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G74" s="6" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="H74" s="6" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="I74" s="6" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="J74" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K74" s="5"/>
       <c r="L74" s="5"/>
@@ -3582,17 +3582,17 @@
     </row>
     <row r="77" spans="1:12" ht="15.5" customHeight="1">
       <c r="A77" s="2" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B77" s="2"/>
       <c r="C77" s="2"/>
-      <c r="D77" s="26" t="s">
-        <v>128</v>
-      </c>
-      <c r="E77" s="27"/>
-      <c r="F77" s="27"/>
-      <c r="G77" s="27"/>
-      <c r="H77" s="28"/>
+      <c r="D77" s="24" t="s">
+        <v>131</v>
+      </c>
+      <c r="E77" s="25"/>
+      <c r="F77" s="25"/>
+      <c r="G77" s="25"/>
+      <c r="H77" s="26"/>
       <c r="I77" s="2"/>
       <c r="J77" s="2"/>
       <c r="K77" s="3"/>
@@ -3622,7 +3622,7 @@
       </c>
       <c r="B79" s="5"/>
       <c r="D79" s="21" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="E79" s="15" t="s">
         <v>17</v>
@@ -3631,16 +3631,16 @@
         <v>18</v>
       </c>
       <c r="G79" s="16" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="H79" s="16" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="I79" s="16" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="J79" s="15" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="K79" s="6"/>
       <c r="L79" s="5"/>
@@ -3677,17 +3677,17 @@
     </row>
     <row r="82" spans="1:12" ht="15.5" customHeight="1">
       <c r="A82" s="2" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="B82" s="2"/>
       <c r="C82" s="2"/>
-      <c r="D82" s="26" t="s">
-        <v>135</v>
-      </c>
-      <c r="E82" s="27"/>
-      <c r="F82" s="27"/>
-      <c r="G82" s="27"/>
-      <c r="H82" s="28"/>
+      <c r="D82" s="24" t="s">
+        <v>138</v>
+      </c>
+      <c r="E82" s="25"/>
+      <c r="F82" s="25"/>
+      <c r="G82" s="25"/>
+      <c r="H82" s="26"/>
       <c r="I82" s="2"/>
       <c r="J82" s="2"/>
       <c r="K82" s="3"/>
@@ -3717,25 +3717,25 @@
       </c>
       <c r="B84" s="5"/>
       <c r="D84" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="E84" s="7" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="F84" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G84" s="6" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="H84" s="6" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="I84" s="6" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="J84" s="7" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="K84" s="5"/>
       <c r="L84" s="5"/>
@@ -3772,17 +3772,17 @@
     </row>
     <row r="87" spans="1:12" ht="15.5" customHeight="1">
       <c r="A87" s="2" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
-      <c r="D87" s="26" t="s">
-        <v>143</v>
-      </c>
-      <c r="E87" s="27"/>
-      <c r="F87" s="27"/>
-      <c r="G87" s="27"/>
-      <c r="H87" s="28"/>
+      <c r="D87" s="24" t="s">
+        <v>146</v>
+      </c>
+      <c r="E87" s="25"/>
+      <c r="F87" s="25"/>
+      <c r="G87" s="25"/>
+      <c r="H87" s="26"/>
       <c r="I87" s="2"/>
       <c r="J87" s="2"/>
       <c r="K87" s="3"/>
@@ -3852,17 +3852,17 @@
     </row>
     <row r="92" spans="1:12" ht="15.5" customHeight="1">
       <c r="A92" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B92" s="2"/>
       <c r="C92" s="2"/>
-      <c r="D92" s="26" t="s">
-        <v>145</v>
-      </c>
-      <c r="E92" s="27"/>
-      <c r="F92" s="27"/>
-      <c r="G92" s="27"/>
-      <c r="H92" s="28"/>
+      <c r="D92" s="24" t="s">
+        <v>148</v>
+      </c>
+      <c r="E92" s="25"/>
+      <c r="F92" s="25"/>
+      <c r="G92" s="25"/>
+      <c r="H92" s="26"/>
       <c r="I92" s="2"/>
       <c r="J92" s="2"/>
       <c r="K92" s="3"/>
@@ -3892,25 +3892,25 @@
       </c>
       <c r="B94" s="5"/>
       <c r="D94" t="s">
-        <v>483</v>
+        <v>149</v>
       </c>
       <c r="E94" s="7" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="F94" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G94" s="6" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="H94" s="6" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="I94" s="6" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="J94" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K94" s="5"/>
       <c r="L94" s="5"/>
@@ -3937,42 +3937,42 @@
       </c>
       <c r="B96" s="5"/>
       <c r="D96" t="s">
-        <v>484</v>
+        <v>154</v>
       </c>
       <c r="E96" s="7" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="F96" s="6" t="s">
         <v>18</v>
       </c>
       <c r="G96" s="6" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="H96" s="6" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="I96" s="6" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="J96" s="7" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="K96" s="5"/>
       <c r="L96" s="5"/>
     </row>
     <row r="97" spans="1:12" ht="15.5" customHeight="1">
       <c r="A97" s="2" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="B97" s="2"/>
       <c r="C97" s="2"/>
-      <c r="D97" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="E97" s="27"/>
-      <c r="F97" s="27"/>
-      <c r="G97" s="27"/>
-      <c r="H97" s="28"/>
+      <c r="D97" s="24" t="s">
+        <v>160</v>
+      </c>
+      <c r="E97" s="25"/>
+      <c r="F97" s="25"/>
+      <c r="G97" s="25"/>
+      <c r="H97" s="26"/>
       <c r="I97" s="2"/>
       <c r="J97" s="2"/>
       <c r="K97" s="3"/>
@@ -4002,25 +4002,25 @@
       </c>
       <c r="B99" s="5"/>
       <c r="D99" t="s">
-        <v>498</v>
+        <v>161</v>
       </c>
       <c r="E99" s="7" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="F99" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G99" s="6" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="H99" s="6" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="I99" s="6" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="J99" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K99" s="5"/>
       <c r="L99" s="5"/>
@@ -4047,42 +4047,42 @@
       </c>
       <c r="B101" s="5"/>
       <c r="D101" t="s">
-        <v>485</v>
+        <v>166</v>
       </c>
       <c r="E101" s="7" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="F101" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G101" s="6" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="H101" s="6" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="I101" s="6" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="J101" s="7" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="K101" s="5"/>
       <c r="L101" s="5"/>
     </row>
     <row r="102" spans="1:12" ht="15.5" customHeight="1">
       <c r="A102" s="2" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="B102" s="2"/>
       <c r="C102" s="2"/>
-      <c r="D102" s="26" t="s">
-        <v>165</v>
-      </c>
-      <c r="E102" s="27"/>
-      <c r="F102" s="27"/>
-      <c r="G102" s="27"/>
-      <c r="H102" s="28"/>
+      <c r="D102" s="24" t="s">
+        <v>172</v>
+      </c>
+      <c r="E102" s="25"/>
+      <c r="F102" s="25"/>
+      <c r="G102" s="25"/>
+      <c r="H102" s="26"/>
       <c r="I102" s="2"/>
       <c r="J102" s="2"/>
       <c r="K102" s="3"/>
@@ -4112,25 +4112,25 @@
       </c>
       <c r="B104" s="5"/>
       <c r="D104" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="E104" s="7" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="F104" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G104" s="6" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="H104" s="6" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="I104" s="6" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="J104" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K104" s="5"/>
       <c r="L104" s="5"/>
@@ -4167,17 +4167,17 @@
     </row>
     <row r="107" spans="1:12" ht="15.5" customHeight="1">
       <c r="A107" s="2" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="B107" s="2"/>
       <c r="C107" s="2"/>
-      <c r="D107" s="26" t="s">
-        <v>172</v>
-      </c>
-      <c r="E107" s="27"/>
-      <c r="F107" s="27"/>
-      <c r="G107" s="27"/>
-      <c r="H107" s="28"/>
+      <c r="D107" s="24" t="s">
+        <v>179</v>
+      </c>
+      <c r="E107" s="25"/>
+      <c r="F107" s="25"/>
+      <c r="G107" s="25"/>
+      <c r="H107" s="26"/>
       <c r="I107" s="2"/>
       <c r="J107" s="2"/>
       <c r="K107" s="3"/>
@@ -4241,17 +4241,17 @@
     </row>
     <row r="112" spans="1:12" ht="15.5" customHeight="1">
       <c r="A112" s="2" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="B112" s="2"/>
       <c r="C112" s="2"/>
-      <c r="D112" s="26" t="s">
-        <v>174</v>
-      </c>
-      <c r="E112" s="27"/>
-      <c r="F112" s="27"/>
-      <c r="G112" s="27"/>
-      <c r="H112" s="28"/>
+      <c r="D112" s="24" t="s">
+        <v>181</v>
+      </c>
+      <c r="E112" s="25"/>
+      <c r="F112" s="25"/>
+      <c r="G112" s="25"/>
+      <c r="H112" s="26"/>
       <c r="I112" s="2"/>
       <c r="J112" s="2"/>
       <c r="K112" s="3"/>
@@ -4281,25 +4281,25 @@
       </c>
       <c r="B114" s="5"/>
       <c r="D114" t="s">
-        <v>486</v>
+        <v>182</v>
       </c>
       <c r="E114" s="7" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="F114" s="6" t="s">
         <v>18</v>
       </c>
       <c r="G114" s="6" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="H114" s="6" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="I114" s="6" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="J114" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K114" s="5"/>
       <c r="L114" s="5"/>
@@ -4336,17 +4336,17 @@
     </row>
     <row r="117" spans="1:12" ht="15.5" customHeight="1">
       <c r="A117" s="2" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="B117" s="2"/>
       <c r="C117" s="2"/>
-      <c r="D117" s="26" t="s">
-        <v>179</v>
-      </c>
-      <c r="E117" s="27"/>
-      <c r="F117" s="27"/>
-      <c r="G117" s="27"/>
-      <c r="H117" s="28"/>
+      <c r="D117" s="24" t="s">
+        <v>187</v>
+      </c>
+      <c r="E117" s="25"/>
+      <c r="F117" s="25"/>
+      <c r="G117" s="25"/>
+      <c r="H117" s="26"/>
       <c r="I117" s="2"/>
       <c r="J117" s="2"/>
       <c r="K117" s="3"/>
@@ -4376,25 +4376,25 @@
       </c>
       <c r="B119" s="5"/>
       <c r="D119" t="s">
-        <v>487</v>
+        <v>188</v>
       </c>
       <c r="E119" s="7" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
       <c r="F119" s="6" t="s">
         <v>18</v>
       </c>
       <c r="G119" s="6" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="H119" s="6" t="s">
-        <v>182</v>
+        <v>191</v>
       </c>
       <c r="I119" s="6" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
       <c r="J119" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K119" s="5"/>
       <c r="L119" s="5"/>
@@ -4431,17 +4431,17 @@
     </row>
     <row r="122" spans="1:12" ht="15.5" customHeight="1">
       <c r="A122" s="2" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="B122" s="2"/>
       <c r="C122" s="2"/>
-      <c r="D122" s="26" t="s">
-        <v>185</v>
-      </c>
-      <c r="E122" s="27"/>
-      <c r="F122" s="27"/>
-      <c r="G122" s="27"/>
-      <c r="H122" s="28"/>
+      <c r="D122" s="24" t="s">
+        <v>194</v>
+      </c>
+      <c r="E122" s="25"/>
+      <c r="F122" s="25"/>
+      <c r="G122" s="25"/>
+      <c r="H122" s="26"/>
       <c r="I122" s="2"/>
       <c r="J122" s="2"/>
       <c r="K122" s="3"/>
@@ -4471,25 +4471,25 @@
       </c>
       <c r="B124" s="5"/>
       <c r="D124" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="E124" s="7" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
       <c r="F124" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G124" s="6" t="s">
-        <v>188</v>
+        <v>197</v>
       </c>
       <c r="H124" s="6" t="s">
-        <v>189</v>
+        <v>198</v>
       </c>
       <c r="I124" s="6" t="s">
-        <v>190</v>
+        <v>199</v>
       </c>
       <c r="J124" s="7" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="K124" s="5"/>
       <c r="L124" s="5"/>
@@ -4526,17 +4526,17 @@
     </row>
     <row r="127" spans="1:12" ht="15.5" customHeight="1">
       <c r="A127" s="2" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
       <c r="B127" s="2"/>
       <c r="C127" s="2"/>
-      <c r="D127" s="26" t="s">
-        <v>192</v>
-      </c>
-      <c r="E127" s="27"/>
-      <c r="F127" s="27"/>
-      <c r="G127" s="27"/>
-      <c r="H127" s="28"/>
+      <c r="D127" s="24" t="s">
+        <v>201</v>
+      </c>
+      <c r="E127" s="25"/>
+      <c r="F127" s="25"/>
+      <c r="G127" s="25"/>
+      <c r="H127" s="26"/>
       <c r="I127" s="2"/>
       <c r="J127" s="2"/>
       <c r="K127" s="3"/>
@@ -4566,22 +4566,22 @@
       </c>
       <c r="B129" s="5"/>
       <c r="D129" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="E129" s="7" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F129" s="6" t="s">
         <v>18</v>
       </c>
       <c r="G129" s="6" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="H129" s="6" t="s">
-        <v>195</v>
+        <v>204</v>
       </c>
       <c r="I129" s="6" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="J129" s="4" t="s">
         <v>22</v>
@@ -4621,17 +4621,17 @@
     </row>
     <row r="132" spans="1:12" ht="15.5" customHeight="1">
       <c r="A132" s="2" t="s">
-        <v>197</v>
+        <v>206</v>
       </c>
       <c r="B132" s="2"/>
       <c r="C132" s="2"/>
-      <c r="D132" s="26" t="s">
-        <v>198</v>
-      </c>
-      <c r="E132" s="27"/>
-      <c r="F132" s="27"/>
-      <c r="G132" s="27"/>
-      <c r="H132" s="28"/>
+      <c r="D132" s="24" t="s">
+        <v>207</v>
+      </c>
+      <c r="E132" s="25"/>
+      <c r="F132" s="25"/>
+      <c r="G132" s="25"/>
+      <c r="H132" s="26"/>
       <c r="I132" s="2"/>
       <c r="J132" s="2"/>
       <c r="K132" s="3"/>
@@ -4661,25 +4661,25 @@
       </c>
       <c r="B134" s="5"/>
       <c r="D134" t="s">
-        <v>199</v>
+        <v>208</v>
       </c>
       <c r="E134" s="7" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F134" s="6" t="s">
         <v>18</v>
       </c>
       <c r="G134" s="6" t="s">
-        <v>200</v>
+        <v>209</v>
       </c>
       <c r="H134" s="6" t="s">
-        <v>201</v>
+        <v>210</v>
       </c>
       <c r="I134" s="6" t="s">
-        <v>202</v>
+        <v>211</v>
       </c>
       <c r="J134" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K134" s="5"/>
       <c r="L134" s="5"/>
@@ -4716,17 +4716,17 @@
     </row>
     <row r="137" spans="1:12" ht="15.5" customHeight="1">
       <c r="A137" s="2" t="s">
-        <v>203</v>
+        <v>212</v>
       </c>
       <c r="B137" s="2"/>
       <c r="C137" s="2"/>
-      <c r="D137" s="26" t="s">
-        <v>204</v>
-      </c>
-      <c r="E137" s="27"/>
-      <c r="F137" s="27"/>
-      <c r="G137" s="27"/>
-      <c r="H137" s="28"/>
+      <c r="D137" s="24" t="s">
+        <v>213</v>
+      </c>
+      <c r="E137" s="25"/>
+      <c r="F137" s="25"/>
+      <c r="G137" s="25"/>
+      <c r="H137" s="26"/>
       <c r="I137" s="2"/>
       <c r="J137" s="2"/>
       <c r="K137" s="3"/>
@@ -4756,25 +4756,25 @@
       </c>
       <c r="B139" s="5"/>
       <c r="D139" t="s">
-        <v>205</v>
+        <v>214</v>
       </c>
       <c r="E139" s="7" t="s">
-        <v>206</v>
+        <v>215</v>
       </c>
       <c r="F139" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G139" s="6" t="s">
-        <v>207</v>
+        <v>216</v>
       </c>
       <c r="H139" s="6" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="I139" s="6" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
       <c r="J139" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K139" s="5"/>
       <c r="L139" s="5"/>
@@ -4811,17 +4811,17 @@
     </row>
     <row r="142" spans="1:12" ht="15.5" customHeight="1">
       <c r="A142" s="2" t="s">
-        <v>210</v>
+        <v>219</v>
       </c>
       <c r="B142" s="2"/>
       <c r="C142" s="2"/>
-      <c r="D142" s="26" t="s">
-        <v>211</v>
-      </c>
-      <c r="E142" s="27"/>
-      <c r="F142" s="27"/>
-      <c r="G142" s="27"/>
-      <c r="H142" s="28"/>
+      <c r="D142" s="24" t="s">
+        <v>220</v>
+      </c>
+      <c r="E142" s="25"/>
+      <c r="F142" s="25"/>
+      <c r="G142" s="25"/>
+      <c r="H142" s="26"/>
       <c r="I142" s="2"/>
       <c r="J142" s="2"/>
       <c r="K142" s="3"/>
@@ -4851,25 +4851,25 @@
       </c>
       <c r="B144" s="5"/>
       <c r="D144" t="s">
-        <v>212</v>
+        <v>221</v>
       </c>
       <c r="E144" s="7" t="s">
-        <v>213</v>
+        <v>222</v>
       </c>
       <c r="F144" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G144" s="6" t="s">
-        <v>214</v>
+        <v>223</v>
       </c>
       <c r="H144" s="6" t="s">
-        <v>215</v>
+        <v>224</v>
       </c>
       <c r="I144" s="6" t="s">
-        <v>216</v>
+        <v>225</v>
       </c>
       <c r="J144" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K144" s="5"/>
       <c r="L144" s="5"/>
@@ -4906,17 +4906,17 @@
     </row>
     <row r="147" spans="1:12" ht="15.5" customHeight="1">
       <c r="A147" s="2" t="s">
-        <v>217</v>
+        <v>226</v>
       </c>
       <c r="B147" s="2"/>
       <c r="C147" s="2"/>
-      <c r="D147" s="26" t="s">
-        <v>218</v>
-      </c>
-      <c r="E147" s="27"/>
-      <c r="F147" s="27"/>
-      <c r="G147" s="27"/>
-      <c r="H147" s="28"/>
+      <c r="D147" s="24" t="s">
+        <v>227</v>
+      </c>
+      <c r="E147" s="25"/>
+      <c r="F147" s="25"/>
+      <c r="G147" s="25"/>
+      <c r="H147" s="26"/>
       <c r="I147" s="2"/>
       <c r="J147" s="2"/>
       <c r="K147" s="3"/>
@@ -4946,25 +4946,25 @@
       </c>
       <c r="B149" s="5"/>
       <c r="D149" t="s">
-        <v>219</v>
+        <v>228</v>
       </c>
       <c r="E149" s="7" t="s">
-        <v>220</v>
+        <v>229</v>
       </c>
       <c r="F149" s="6" t="s">
         <v>18</v>
       </c>
       <c r="G149" s="6" t="s">
-        <v>221</v>
+        <v>230</v>
       </c>
       <c r="H149" s="6" t="s">
-        <v>222</v>
+        <v>231</v>
       </c>
       <c r="I149" s="6" t="s">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="J149" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K149" s="5"/>
       <c r="L149" s="5"/>
@@ -5001,17 +5001,17 @@
     </row>
     <row r="152" spans="1:12" ht="15.5" customHeight="1">
       <c r="A152" s="2" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="B152" s="2"/>
       <c r="C152" s="2"/>
-      <c r="D152" s="26" t="s">
-        <v>225</v>
-      </c>
-      <c r="E152" s="27"/>
-      <c r="F152" s="27"/>
-      <c r="G152" s="27"/>
-      <c r="H152" s="28"/>
+      <c r="D152" s="24" t="s">
+        <v>234</v>
+      </c>
+      <c r="E152" s="25"/>
+      <c r="F152" s="25"/>
+      <c r="G152" s="25"/>
+      <c r="H152" s="26"/>
       <c r="I152" s="2"/>
       <c r="J152" s="2"/>
       <c r="K152" s="3"/>
@@ -5041,7 +5041,7 @@
       </c>
       <c r="B154" s="5"/>
       <c r="D154" s="21" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="E154" s="15" t="s">
         <v>17</v>
@@ -5050,16 +5050,16 @@
         <v>18</v>
       </c>
       <c r="G154" s="16" t="s">
-        <v>227</v>
+        <v>236</v>
       </c>
       <c r="H154" s="16" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="I154" s="16" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="J154" s="15" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K154" s="5"/>
       <c r="L154" s="5"/>
@@ -5096,17 +5096,17 @@
     </row>
     <row r="157" spans="1:12" ht="15.5" customHeight="1">
       <c r="A157" s="2" t="s">
-        <v>230</v>
+        <v>239</v>
       </c>
       <c r="B157" s="2"/>
       <c r="C157" s="2"/>
-      <c r="D157" s="26" t="s">
-        <v>231</v>
-      </c>
-      <c r="E157" s="27"/>
-      <c r="F157" s="27"/>
-      <c r="G157" s="27"/>
-      <c r="H157" s="28"/>
+      <c r="D157" s="24" t="s">
+        <v>240</v>
+      </c>
+      <c r="E157" s="25"/>
+      <c r="F157" s="25"/>
+      <c r="G157" s="25"/>
+      <c r="H157" s="26"/>
       <c r="I157" s="2"/>
       <c r="J157" s="2"/>
       <c r="K157" s="3"/>
@@ -5136,25 +5136,25 @@
       </c>
       <c r="B159" s="5"/>
       <c r="D159" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="E159" s="12" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
       <c r="F159" s="9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G159" s="7" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="H159" s="6" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
       <c r="I159" s="6" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="J159" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="K159" s="5"/>
       <c r="L159" s="5"/>
@@ -5191,17 +5191,17 @@
     </row>
     <row r="162" spans="1:12" ht="15.5" customHeight="1">
       <c r="A162" s="2" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="B162" s="2"/>
       <c r="C162" s="2"/>
-      <c r="D162" s="26" t="s">
-        <v>238</v>
-      </c>
-      <c r="E162" s="27"/>
-      <c r="F162" s="27"/>
-      <c r="G162" s="27"/>
-      <c r="H162" s="28"/>
+      <c r="D162" s="24" t="s">
+        <v>247</v>
+      </c>
+      <c r="E162" s="25"/>
+      <c r="F162" s="25"/>
+      <c r="G162" s="25"/>
+      <c r="H162" s="26"/>
       <c r="I162" s="2"/>
       <c r="J162" s="2"/>
       <c r="K162" s="3"/>
@@ -5231,25 +5231,25 @@
       </c>
       <c r="B164" s="5"/>
       <c r="D164" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="E164" s="7" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
       <c r="F164" s="6" t="s">
         <v>18</v>
       </c>
       <c r="G164" s="6" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
       <c r="H164" s="6" t="s">
-        <v>242</v>
+        <v>251</v>
       </c>
       <c r="I164" s="6" t="s">
-        <v>243</v>
+        <v>252</v>
       </c>
       <c r="J164" s="7" t="s">
-        <v>244</v>
+        <v>253</v>
       </c>
       <c r="K164" s="5"/>
       <c r="L164" s="5"/>
@@ -5286,17 +5286,17 @@
     </row>
     <row r="167" spans="1:12" ht="15.5" customHeight="1">
       <c r="A167" s="2" t="s">
-        <v>245</v>
+        <v>254</v>
       </c>
       <c r="B167" s="2"/>
       <c r="C167" s="2"/>
-      <c r="D167" s="26" t="s">
-        <v>246</v>
-      </c>
-      <c r="E167" s="27"/>
-      <c r="F167" s="27"/>
-      <c r="G167" s="27"/>
-      <c r="H167" s="28"/>
+      <c r="D167" s="24" t="s">
+        <v>255</v>
+      </c>
+      <c r="E167" s="25"/>
+      <c r="F167" s="25"/>
+      <c r="G167" s="25"/>
+      <c r="H167" s="26"/>
       <c r="I167" s="2"/>
       <c r="J167" s="2"/>
       <c r="K167" s="3"/>
@@ -5326,25 +5326,25 @@
       </c>
       <c r="B169" s="5"/>
       <c r="D169" t="s">
-        <v>247</v>
+        <v>256</v>
       </c>
       <c r="E169" s="7" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="F169" s="6" t="s">
         <v>18</v>
       </c>
       <c r="G169" s="6" t="s">
-        <v>249</v>
+        <v>258</v>
       </c>
       <c r="H169" s="6" t="s">
-        <v>250</v>
+        <v>259</v>
       </c>
       <c r="I169" s="6" t="s">
-        <v>251</v>
+        <v>260</v>
       </c>
       <c r="J169" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K169" s="5"/>
       <c r="L169" s="5"/>
@@ -5381,17 +5381,17 @@
     </row>
     <row r="172" spans="1:12" ht="15.5" customHeight="1">
       <c r="A172" s="2" t="s">
-        <v>252</v>
+        <v>261</v>
       </c>
       <c r="B172" s="2"/>
       <c r="C172" s="2"/>
-      <c r="D172" s="26" t="s">
-        <v>253</v>
-      </c>
-      <c r="E172" s="27"/>
-      <c r="F172" s="27"/>
-      <c r="G172" s="27"/>
-      <c r="H172" s="28"/>
+      <c r="D172" s="24" t="s">
+        <v>262</v>
+      </c>
+      <c r="E172" s="25"/>
+      <c r="F172" s="25"/>
+      <c r="G172" s="25"/>
+      <c r="H172" s="26"/>
       <c r="I172" s="2"/>
       <c r="J172" s="2"/>
       <c r="K172" s="3"/>
@@ -5421,25 +5421,25 @@
       </c>
       <c r="B174" s="5"/>
       <c r="D174" t="s">
-        <v>488</v>
+        <v>263</v>
       </c>
       <c r="E174" s="7" t="s">
-        <v>254</v>
+        <v>264</v>
       </c>
       <c r="F174" s="6" t="s">
         <v>18</v>
       </c>
       <c r="G174" s="6" t="s">
-        <v>255</v>
+        <v>265</v>
       </c>
       <c r="H174" s="6" t="s">
-        <v>256</v>
+        <v>266</v>
       </c>
       <c r="I174" s="6" t="s">
-        <v>257</v>
+        <v>267</v>
       </c>
       <c r="J174" s="7" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="K174" s="5"/>
       <c r="L174" s="5"/>
@@ -5476,17 +5476,17 @@
     </row>
     <row r="177" spans="1:12" ht="15.5" customHeight="1">
       <c r="A177" s="2" t="s">
-        <v>258</v>
+        <v>268</v>
       </c>
       <c r="B177" s="2"/>
       <c r="C177" s="2"/>
-      <c r="D177" s="26" t="s">
-        <v>259</v>
-      </c>
-      <c r="E177" s="27"/>
-      <c r="F177" s="27"/>
-      <c r="G177" s="27"/>
-      <c r="H177" s="28"/>
+      <c r="D177" s="24" t="s">
+        <v>269</v>
+      </c>
+      <c r="E177" s="25"/>
+      <c r="F177" s="25"/>
+      <c r="G177" s="25"/>
+      <c r="H177" s="26"/>
       <c r="I177" s="2"/>
       <c r="J177" s="2"/>
       <c r="K177" s="3"/>
@@ -5514,22 +5514,22 @@
       </c>
       <c r="B179" s="5"/>
       <c r="D179" t="s">
-        <v>489</v>
+        <v>270</v>
       </c>
       <c r="E179" s="7" t="s">
-        <v>260</v>
+        <v>271</v>
       </c>
       <c r="F179" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G179" s="6" t="s">
-        <v>261</v>
+        <v>272</v>
       </c>
       <c r="H179" s="6" t="s">
-        <v>262</v>
+        <v>273</v>
       </c>
       <c r="I179" s="6" t="s">
-        <v>263</v>
+        <v>274</v>
       </c>
       <c r="J179" s="15" t="s">
         <v>22</v>
@@ -5569,17 +5569,17 @@
     </row>
     <row r="182" spans="1:12" ht="15.5" customHeight="1">
       <c r="A182" s="2" t="s">
-        <v>264</v>
+        <v>275</v>
       </c>
       <c r="B182" s="2"/>
       <c r="C182" s="2"/>
-      <c r="D182" s="26" t="s">
-        <v>265</v>
-      </c>
-      <c r="E182" s="27"/>
-      <c r="F182" s="27"/>
-      <c r="G182" s="27"/>
-      <c r="H182" s="28"/>
+      <c r="D182" s="24" t="s">
+        <v>276</v>
+      </c>
+      <c r="E182" s="25"/>
+      <c r="F182" s="25"/>
+      <c r="G182" s="25"/>
+      <c r="H182" s="26"/>
       <c r="I182" s="2"/>
       <c r="J182" s="2"/>
       <c r="K182" s="3"/>
@@ -5609,25 +5609,25 @@
       </c>
       <c r="B184" s="5"/>
       <c r="D184" t="s">
-        <v>266</v>
+        <v>277</v>
       </c>
       <c r="E184" s="7" t="s">
-        <v>267</v>
+        <v>278</v>
       </c>
       <c r="F184" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G184" s="6" t="s">
-        <v>268</v>
+        <v>279</v>
       </c>
       <c r="H184" s="6" t="s">
-        <v>269</v>
+        <v>280</v>
       </c>
       <c r="I184" s="6" t="s">
-        <v>270</v>
+        <v>281</v>
       </c>
       <c r="J184" s="7" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="K184" s="5"/>
       <c r="L184" s="5"/>
@@ -5664,17 +5664,17 @@
     </row>
     <row r="187" spans="1:12" ht="15.5" customHeight="1">
       <c r="A187" s="2" t="s">
-        <v>271</v>
+        <v>282</v>
       </c>
       <c r="B187" s="2"/>
       <c r="C187" s="2"/>
-      <c r="D187" s="26" t="s">
-        <v>272</v>
-      </c>
-      <c r="E187" s="27"/>
-      <c r="F187" s="27"/>
-      <c r="G187" s="27"/>
-      <c r="H187" s="28"/>
+      <c r="D187" s="24" t="s">
+        <v>283</v>
+      </c>
+      <c r="E187" s="25"/>
+      <c r="F187" s="25"/>
+      <c r="G187" s="25"/>
+      <c r="H187" s="26"/>
       <c r="I187" s="2"/>
       <c r="J187" s="2"/>
       <c r="K187" s="3"/>
@@ -5704,25 +5704,25 @@
       </c>
       <c r="B189" s="5"/>
       <c r="D189" t="s">
-        <v>273</v>
+        <v>284</v>
       </c>
       <c r="E189" s="7" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="F189" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G189" s="6" t="s">
-        <v>274</v>
+        <v>285</v>
       </c>
       <c r="H189" s="6" t="s">
-        <v>275</v>
+        <v>286</v>
       </c>
       <c r="I189" s="6" t="s">
-        <v>276</v>
+        <v>287</v>
       </c>
       <c r="J189" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K189" s="5"/>
       <c r="L189" s="5"/>
@@ -5749,42 +5749,42 @@
       </c>
       <c r="B191" s="5"/>
       <c r="D191" t="s">
-        <v>277</v>
+        <v>288</v>
       </c>
       <c r="E191" s="7" t="s">
-        <v>267</v>
+        <v>278</v>
       </c>
       <c r="F191" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G191" s="6" t="s">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="H191" s="6" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="I191" s="6" t="s">
-        <v>280</v>
+        <v>291</v>
       </c>
       <c r="J191" s="7" t="s">
-        <v>281</v>
+        <v>292</v>
       </c>
       <c r="K191" s="5"/>
       <c r="L191" s="5"/>
     </row>
     <row r="192" spans="1:12" ht="15.5" customHeight="1">
       <c r="A192" s="2" t="s">
-        <v>282</v>
+        <v>293</v>
       </c>
       <c r="B192" s="2"/>
       <c r="C192" s="2"/>
-      <c r="D192" s="26" t="s">
-        <v>283</v>
-      </c>
-      <c r="E192" s="27"/>
-      <c r="F192" s="27"/>
-      <c r="G192" s="27"/>
-      <c r="H192" s="28"/>
+      <c r="D192" s="24" t="s">
+        <v>294</v>
+      </c>
+      <c r="E192" s="25"/>
+      <c r="F192" s="25"/>
+      <c r="G192" s="25"/>
+      <c r="H192" s="26"/>
       <c r="I192" s="2"/>
       <c r="J192" s="2"/>
       <c r="K192" s="3"/>
@@ -5814,25 +5814,25 @@
       </c>
       <c r="B194" s="5"/>
       <c r="D194" s="21" t="s">
-        <v>284</v>
+        <v>295</v>
       </c>
       <c r="E194" s="15" t="s">
-        <v>285</v>
+        <v>296</v>
       </c>
       <c r="F194" s="16" t="s">
         <v>18</v>
       </c>
       <c r="G194" s="16" t="s">
-        <v>286</v>
+        <v>297</v>
       </c>
       <c r="H194" s="20" t="s">
-        <v>287</v>
+        <v>298</v>
       </c>
       <c r="I194" s="16" t="s">
-        <v>288</v>
+        <v>299</v>
       </c>
       <c r="J194" s="16" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="K194" s="5"/>
       <c r="L194" s="5"/>
@@ -5869,17 +5869,17 @@
     </row>
     <row r="197" spans="1:12" ht="15.5" customHeight="1">
       <c r="A197" s="2" t="s">
-        <v>289</v>
+        <v>300</v>
       </c>
       <c r="B197" s="2"/>
       <c r="C197" s="2"/>
-      <c r="D197" s="26" t="s">
-        <v>290</v>
-      </c>
-      <c r="E197" s="27"/>
-      <c r="F197" s="27"/>
-      <c r="G197" s="27"/>
-      <c r="H197" s="28"/>
+      <c r="D197" s="24" t="s">
+        <v>301</v>
+      </c>
+      <c r="E197" s="25"/>
+      <c r="F197" s="25"/>
+      <c r="G197" s="25"/>
+      <c r="H197" s="26"/>
       <c r="I197" s="2"/>
       <c r="J197" s="2"/>
       <c r="K197" s="3"/>
@@ -5909,25 +5909,25 @@
       </c>
       <c r="B199" s="5"/>
       <c r="D199" t="s">
-        <v>490</v>
+        <v>302</v>
       </c>
       <c r="E199" s="12" t="s">
-        <v>291</v>
+        <v>303</v>
       </c>
       <c r="F199" s="9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G199" s="7" t="s">
-        <v>292</v>
+        <v>304</v>
       </c>
       <c r="H199" s="6" t="s">
-        <v>293</v>
+        <v>305</v>
       </c>
       <c r="I199" s="6" t="s">
-        <v>294</v>
+        <v>306</v>
       </c>
       <c r="J199" s="7" t="s">
-        <v>295</v>
+        <v>307</v>
       </c>
       <c r="K199" s="5"/>
       <c r="L199" s="5"/>
@@ -5964,17 +5964,17 @@
     </row>
     <row r="202" spans="1:12" ht="15.5" customHeight="1">
       <c r="A202" s="2" t="s">
-        <v>296</v>
+        <v>308</v>
       </c>
       <c r="B202" s="2"/>
       <c r="C202" s="2"/>
-      <c r="D202" s="26" t="s">
-        <v>297</v>
-      </c>
-      <c r="E202" s="27"/>
-      <c r="F202" s="27"/>
-      <c r="G202" s="27"/>
-      <c r="H202" s="28"/>
+      <c r="D202" s="24" t="s">
+        <v>309</v>
+      </c>
+      <c r="E202" s="25"/>
+      <c r="F202" s="25"/>
+      <c r="G202" s="25"/>
+      <c r="H202" s="26"/>
       <c r="I202" s="2"/>
       <c r="J202" s="2"/>
       <c r="K202" s="3"/>
@@ -6004,25 +6004,25 @@
       </c>
       <c r="B204" s="5"/>
       <c r="D204" s="21" t="s">
-        <v>298</v>
+        <v>310</v>
       </c>
       <c r="E204" s="15" t="s">
         <v>17</v>
       </c>
       <c r="F204" s="16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G204" s="16" t="s">
-        <v>299</v>
+        <v>311</v>
       </c>
       <c r="H204" s="16" t="s">
-        <v>300</v>
+        <v>312</v>
       </c>
       <c r="I204" s="16" t="s">
-        <v>301</v>
+        <v>313</v>
       </c>
       <c r="J204" s="15" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="K204" s="5"/>
       <c r="L204" s="5"/>
@@ -6059,17 +6059,17 @@
     </row>
     <row r="207" spans="1:12" ht="15.5" customHeight="1">
       <c r="A207" s="2" t="s">
-        <v>302</v>
+        <v>314</v>
       </c>
       <c r="B207" s="2"/>
       <c r="C207" s="2"/>
-      <c r="D207" s="26" t="s">
-        <v>303</v>
-      </c>
-      <c r="E207" s="27"/>
-      <c r="F207" s="27"/>
-      <c r="G207" s="27"/>
-      <c r="H207" s="28"/>
+      <c r="D207" s="24" t="s">
+        <v>315</v>
+      </c>
+      <c r="E207" s="25"/>
+      <c r="F207" s="25"/>
+      <c r="G207" s="25"/>
+      <c r="H207" s="26"/>
       <c r="I207" s="2"/>
       <c r="J207" s="2"/>
       <c r="K207" s="3"/>
@@ -6099,22 +6099,22 @@
       </c>
       <c r="B209" s="5"/>
       <c r="D209" t="s">
-        <v>304</v>
+        <v>316</v>
       </c>
       <c r="E209" s="7" t="s">
-        <v>305</v>
+        <v>317</v>
       </c>
       <c r="F209" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G209" s="6" t="s">
-        <v>306</v>
+        <v>318</v>
       </c>
       <c r="H209" s="6" t="s">
-        <v>307</v>
+        <v>319</v>
       </c>
       <c r="I209" s="6" t="s">
-        <v>308</v>
+        <v>320</v>
       </c>
       <c r="J209" s="15" t="s">
         <v>22</v>
@@ -6154,17 +6154,17 @@
     </row>
     <row r="212" spans="1:12" ht="15.5" customHeight="1">
       <c r="A212" s="2" t="s">
-        <v>309</v>
+        <v>321</v>
       </c>
       <c r="B212" s="2"/>
       <c r="C212" s="2"/>
-      <c r="D212" s="26" t="s">
-        <v>310</v>
-      </c>
-      <c r="E212" s="27"/>
-      <c r="F212" s="27"/>
-      <c r="G212" s="27"/>
-      <c r="H212" s="28"/>
+      <c r="D212" s="24" t="s">
+        <v>322</v>
+      </c>
+      <c r="E212" s="25"/>
+      <c r="F212" s="25"/>
+      <c r="G212" s="25"/>
+      <c r="H212" s="26"/>
       <c r="I212" s="2"/>
       <c r="J212" s="2"/>
       <c r="K212" s="3"/>
@@ -6194,25 +6194,25 @@
       </c>
       <c r="B214" s="5"/>
       <c r="D214" t="s">
-        <v>311</v>
+        <v>323</v>
       </c>
       <c r="E214" s="7" t="s">
-        <v>312</v>
+        <v>324</v>
       </c>
       <c r="F214" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G214" s="6" t="s">
-        <v>313</v>
+        <v>325</v>
       </c>
       <c r="H214" s="6" t="s">
-        <v>314</v>
+        <v>326</v>
       </c>
       <c r="I214" s="6" t="s">
-        <v>315</v>
+        <v>327</v>
       </c>
       <c r="J214" s="7" t="s">
-        <v>316</v>
+        <v>328</v>
       </c>
       <c r="K214" s="5"/>
       <c r="L214" s="5"/>
@@ -6249,17 +6249,17 @@
     </row>
     <row r="217" spans="1:12" ht="15.5" customHeight="1">
       <c r="A217" s="2" t="s">
-        <v>317</v>
+        <v>329</v>
       </c>
       <c r="B217" s="2"/>
       <c r="C217" s="2"/>
-      <c r="D217" s="26" t="s">
-        <v>318</v>
-      </c>
-      <c r="E217" s="27"/>
-      <c r="F217" s="27"/>
-      <c r="G217" s="27"/>
-      <c r="H217" s="28"/>
+      <c r="D217" s="24" t="s">
+        <v>330</v>
+      </c>
+      <c r="E217" s="25"/>
+      <c r="F217" s="25"/>
+      <c r="G217" s="25"/>
+      <c r="H217" s="26"/>
       <c r="I217" s="2"/>
       <c r="J217" s="2"/>
       <c r="K217" s="3"/>
@@ -6289,25 +6289,25 @@
       </c>
       <c r="B219" s="5"/>
       <c r="D219" t="s">
-        <v>319</v>
+        <v>331</v>
       </c>
       <c r="E219" s="7" t="s">
-        <v>260</v>
+        <v>271</v>
       </c>
       <c r="F219" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G219" s="6" t="s">
-        <v>320</v>
+        <v>332</v>
       </c>
       <c r="H219" s="6" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
       <c r="I219" s="6" t="s">
-        <v>322</v>
+        <v>334</v>
       </c>
       <c r="J219" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K219" s="5"/>
       <c r="L219" s="5"/>
@@ -6344,17 +6344,17 @@
     </row>
     <row r="222" spans="1:12" ht="15.5" customHeight="1">
       <c r="A222" s="2" t="s">
-        <v>323</v>
+        <v>335</v>
       </c>
       <c r="B222" s="2"/>
       <c r="C222" s="2"/>
-      <c r="D222" s="26" t="s">
-        <v>324</v>
-      </c>
-      <c r="E222" s="27"/>
-      <c r="F222" s="27"/>
-      <c r="G222" s="27"/>
-      <c r="H222" s="28"/>
+      <c r="D222" s="24" t="s">
+        <v>336</v>
+      </c>
+      <c r="E222" s="25"/>
+      <c r="F222" s="25"/>
+      <c r="G222" s="25"/>
+      <c r="H222" s="26"/>
       <c r="I222" s="2"/>
       <c r="J222" s="2"/>
       <c r="K222" s="3"/>
@@ -6384,7 +6384,7 @@
       </c>
       <c r="B224" s="5"/>
       <c r="D224" s="21" t="s">
-        <v>325</v>
+        <v>337</v>
       </c>
       <c r="E224" s="15" t="s">
         <v>17</v>
@@ -6393,13 +6393,13 @@
         <v>18</v>
       </c>
       <c r="G224" s="16" t="s">
-        <v>326</v>
+        <v>338</v>
       </c>
       <c r="H224" s="16" t="s">
-        <v>327</v>
+        <v>339</v>
       </c>
       <c r="I224" s="16" t="s">
-        <v>328</v>
+        <v>340</v>
       </c>
       <c r="J224" s="15" t="s">
         <v>22</v>
@@ -6439,17 +6439,17 @@
     </row>
     <row r="227" spans="1:12" ht="15.5" customHeight="1">
       <c r="A227" s="2" t="s">
-        <v>329</v>
+        <v>341</v>
       </c>
       <c r="B227" s="2"/>
       <c r="C227" s="2"/>
-      <c r="D227" s="26" t="s">
-        <v>330</v>
-      </c>
-      <c r="E227" s="27"/>
-      <c r="F227" s="27"/>
-      <c r="G227" s="27"/>
-      <c r="H227" s="28"/>
+      <c r="D227" s="24" t="s">
+        <v>342</v>
+      </c>
+      <c r="E227" s="25"/>
+      <c r="F227" s="25"/>
+      <c r="G227" s="25"/>
+      <c r="H227" s="26"/>
       <c r="I227" s="2"/>
       <c r="J227" s="2"/>
       <c r="K227" s="3"/>
@@ -6479,7 +6479,7 @@
       </c>
       <c r="B229" s="5"/>
       <c r="D229" s="21" t="s">
-        <v>331</v>
+        <v>343</v>
       </c>
       <c r="E229" s="15" t="s">
         <v>17</v>
@@ -6488,16 +6488,16 @@
         <v>18</v>
       </c>
       <c r="G229" s="16" t="s">
-        <v>332</v>
+        <v>344</v>
       </c>
       <c r="H229" s="16" t="s">
-        <v>333</v>
+        <v>345</v>
       </c>
       <c r="I229" s="16" t="s">
-        <v>334</v>
+        <v>346</v>
       </c>
       <c r="J229" s="15" t="s">
-        <v>281</v>
+        <v>292</v>
       </c>
       <c r="K229" s="6"/>
       <c r="L229" s="5"/>
@@ -6524,7 +6524,7 @@
       </c>
       <c r="B231" s="5"/>
       <c r="D231" s="21" t="s">
-        <v>335</v>
+        <v>347</v>
       </c>
       <c r="E231" s="15" t="s">
         <v>17</v>
@@ -6533,33 +6533,33 @@
         <v>18</v>
       </c>
       <c r="G231" s="16" t="s">
-        <v>336</v>
+        <v>348</v>
       </c>
       <c r="H231" s="16" t="s">
-        <v>337</v>
+        <v>349</v>
       </c>
       <c r="I231" s="16" t="s">
-        <v>338</v>
+        <v>350</v>
       </c>
       <c r="J231" s="15" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="K231" s="6"/>
       <c r="L231" s="5"/>
     </row>
     <row r="232" spans="1:12" ht="15.5" customHeight="1">
       <c r="A232" s="2" t="s">
-        <v>339</v>
+        <v>351</v>
       </c>
       <c r="B232" s="2"/>
       <c r="C232" s="2"/>
-      <c r="D232" s="26" t="s">
-        <v>340</v>
-      </c>
-      <c r="E232" s="27"/>
-      <c r="F232" s="27"/>
-      <c r="G232" s="27"/>
-      <c r="H232" s="28"/>
+      <c r="D232" s="24" t="s">
+        <v>352</v>
+      </c>
+      <c r="E232" s="25"/>
+      <c r="F232" s="25"/>
+      <c r="G232" s="25"/>
+      <c r="H232" s="26"/>
       <c r="I232" s="2"/>
       <c r="J232" s="2"/>
       <c r="K232" s="3"/>
@@ -6589,25 +6589,25 @@
       </c>
       <c r="B234" s="5"/>
       <c r="D234" t="s">
-        <v>341</v>
+        <v>353</v>
       </c>
       <c r="E234" s="7" t="s">
-        <v>342</v>
+        <v>354</v>
       </c>
       <c r="F234" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G234" s="6" t="s">
-        <v>343</v>
+        <v>355</v>
       </c>
       <c r="H234" s="6" t="s">
-        <v>344</v>
+        <v>356</v>
       </c>
       <c r="I234" s="6" t="s">
-        <v>345</v>
+        <v>357</v>
       </c>
       <c r="J234" s="7" t="s">
-        <v>244</v>
+        <v>253</v>
       </c>
       <c r="K234" s="5"/>
       <c r="L234" s="5"/>
@@ -6644,17 +6644,17 @@
     </row>
     <row r="237" spans="1:12" ht="15.5" customHeight="1">
       <c r="A237" s="2" t="s">
-        <v>346</v>
+        <v>358</v>
       </c>
       <c r="B237" s="2"/>
       <c r="C237" s="2"/>
-      <c r="D237" s="26" t="s">
-        <v>347</v>
-      </c>
-      <c r="E237" s="27"/>
-      <c r="F237" s="27"/>
-      <c r="G237" s="27"/>
-      <c r="H237" s="28"/>
+      <c r="D237" s="24" t="s">
+        <v>359</v>
+      </c>
+      <c r="E237" s="25"/>
+      <c r="F237" s="25"/>
+      <c r="G237" s="25"/>
+      <c r="H237" s="26"/>
       <c r="I237" s="2"/>
       <c r="J237" s="2"/>
       <c r="K237" s="3"/>
@@ -6684,25 +6684,25 @@
       </c>
       <c r="B239" s="5"/>
       <c r="D239" t="s">
-        <v>348</v>
+        <v>360</v>
       </c>
       <c r="E239" s="7" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
       <c r="F239" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G239" s="6" t="s">
-        <v>349</v>
+        <v>361</v>
       </c>
       <c r="H239" s="6" t="s">
-        <v>350</v>
+        <v>362</v>
       </c>
       <c r="I239" s="6" t="s">
-        <v>351</v>
+        <v>363</v>
       </c>
       <c r="J239" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K239" s="5"/>
       <c r="L239" s="5"/>
@@ -6739,17 +6739,17 @@
     </row>
     <row r="242" spans="1:12" ht="15.5" customHeight="1">
       <c r="A242" s="2" t="s">
-        <v>352</v>
+        <v>364</v>
       </c>
       <c r="B242" s="2"/>
       <c r="C242" s="2"/>
-      <c r="D242" s="26" t="s">
-        <v>353</v>
-      </c>
-      <c r="E242" s="27"/>
-      <c r="F242" s="27"/>
-      <c r="G242" s="27"/>
-      <c r="H242" s="28"/>
+      <c r="D242" s="24" t="s">
+        <v>365</v>
+      </c>
+      <c r="E242" s="25"/>
+      <c r="F242" s="25"/>
+      <c r="G242" s="25"/>
+      <c r="H242" s="26"/>
       <c r="I242" s="2"/>
       <c r="J242" s="2"/>
       <c r="K242" s="3"/>
@@ -6779,25 +6779,25 @@
       </c>
       <c r="B244" s="5"/>
       <c r="D244" t="s">
-        <v>354</v>
+        <v>366</v>
       </c>
       <c r="E244" s="7" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="F244" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G244" s="6" t="s">
-        <v>355</v>
+        <v>367</v>
       </c>
       <c r="H244" s="6" t="s">
-        <v>356</v>
+        <v>368</v>
       </c>
       <c r="I244" s="6" t="s">
-        <v>357</v>
+        <v>369</v>
       </c>
       <c r="J244" s="7" t="s">
-        <v>358</v>
+        <v>370</v>
       </c>
       <c r="K244" s="5"/>
       <c r="L244" s="5"/>
@@ -6834,17 +6834,17 @@
     </row>
     <row r="247" spans="1:12" ht="15.5" customHeight="1">
       <c r="A247" s="2" t="s">
-        <v>359</v>
+        <v>371</v>
       </c>
       <c r="B247" s="2"/>
       <c r="C247" s="2"/>
-      <c r="D247" s="26" t="s">
-        <v>360</v>
-      </c>
-      <c r="E247" s="27"/>
-      <c r="F247" s="27"/>
-      <c r="G247" s="27"/>
-      <c r="H247" s="28"/>
+      <c r="D247" s="24" t="s">
+        <v>372</v>
+      </c>
+      <c r="E247" s="25"/>
+      <c r="F247" s="25"/>
+      <c r="G247" s="25"/>
+      <c r="H247" s="26"/>
       <c r="I247" s="2"/>
       <c r="J247" s="2"/>
       <c r="K247" s="3"/>
@@ -6874,22 +6874,22 @@
       </c>
       <c r="B249" s="5"/>
       <c r="D249" t="s">
-        <v>361</v>
+        <v>373</v>
       </c>
       <c r="E249" s="7" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
       <c r="F249" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G249" s="6" t="s">
-        <v>362</v>
+        <v>374</v>
       </c>
       <c r="H249" s="6" t="s">
-        <v>363</v>
+        <v>375</v>
       </c>
       <c r="I249" s="6" t="s">
-        <v>364</v>
+        <v>376</v>
       </c>
       <c r="J249" s="15" t="s">
         <v>22</v>
@@ -6929,17 +6929,17 @@
     </row>
     <row r="252" spans="1:12" ht="15.5" customHeight="1">
       <c r="A252" s="2" t="s">
-        <v>365</v>
+        <v>377</v>
       </c>
       <c r="B252" s="2"/>
       <c r="C252" s="2"/>
-      <c r="D252" s="26" t="s">
-        <v>366</v>
-      </c>
-      <c r="E252" s="27"/>
-      <c r="F252" s="27"/>
-      <c r="G252" s="27"/>
-      <c r="H252" s="28"/>
+      <c r="D252" s="24" t="s">
+        <v>378</v>
+      </c>
+      <c r="E252" s="25"/>
+      <c r="F252" s="25"/>
+      <c r="G252" s="25"/>
+      <c r="H252" s="26"/>
       <c r="I252" s="2"/>
       <c r="J252" s="2"/>
       <c r="K252" s="3"/>
@@ -6969,25 +6969,25 @@
       </c>
       <c r="B254" s="5"/>
       <c r="D254" t="s">
-        <v>491</v>
+        <v>379</v>
       </c>
       <c r="E254" s="7" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F254" s="6" t="s">
         <v>18</v>
       </c>
       <c r="G254" s="6" t="s">
-        <v>367</v>
+        <v>380</v>
       </c>
       <c r="H254" s="6" t="s">
-        <v>368</v>
+        <v>381</v>
       </c>
       <c r="I254" s="6" t="s">
-        <v>369</v>
+        <v>382</v>
       </c>
       <c r="J254" s="7" t="s">
-        <v>358</v>
+        <v>370</v>
       </c>
       <c r="K254" s="5"/>
       <c r="L254" s="5"/>
@@ -7024,17 +7024,17 @@
     </row>
     <row r="257" spans="1:12" ht="15.5" customHeight="1">
       <c r="A257" s="2" t="s">
-        <v>370</v>
+        <v>383</v>
       </c>
       <c r="B257" s="2"/>
       <c r="C257" s="2"/>
-      <c r="D257" s="26" t="s">
-        <v>371</v>
-      </c>
-      <c r="E257" s="27"/>
-      <c r="F257" s="27"/>
-      <c r="G257" s="27"/>
-      <c r="H257" s="28"/>
+      <c r="D257" s="24" t="s">
+        <v>384</v>
+      </c>
+      <c r="E257" s="25"/>
+      <c r="F257" s="25"/>
+      <c r="G257" s="25"/>
+      <c r="H257" s="26"/>
       <c r="I257" s="2"/>
       <c r="J257" s="2"/>
       <c r="K257" s="3"/>
@@ -7064,25 +7064,25 @@
       </c>
       <c r="B259" s="5"/>
       <c r="D259" t="s">
-        <v>492</v>
+        <v>385</v>
       </c>
       <c r="E259" s="7" t="s">
-        <v>372</v>
+        <v>386</v>
       </c>
       <c r="F259" s="6" t="s">
         <v>18</v>
       </c>
       <c r="G259" s="6" t="s">
-        <v>373</v>
+        <v>387</v>
       </c>
       <c r="H259" s="6" t="s">
-        <v>374</v>
+        <v>388</v>
       </c>
       <c r="I259" s="6" t="s">
-        <v>375</v>
+        <v>389</v>
       </c>
       <c r="J259" s="7" t="s">
-        <v>376</v>
+        <v>390</v>
       </c>
       <c r="K259" s="5"/>
       <c r="L259" s="5"/>
@@ -7113,17 +7113,17 @@
     </row>
     <row r="262" spans="1:12" ht="15.5" customHeight="1">
       <c r="A262" s="2" t="s">
-        <v>377</v>
+        <v>391</v>
       </c>
       <c r="B262" s="2"/>
       <c r="C262" s="2"/>
-      <c r="D262" s="26" t="s">
-        <v>378</v>
-      </c>
-      <c r="E262" s="27"/>
-      <c r="F262" s="27"/>
-      <c r="G262" s="27"/>
-      <c r="H262" s="28"/>
+      <c r="D262" s="24" t="s">
+        <v>392</v>
+      </c>
+      <c r="E262" s="25"/>
+      <c r="F262" s="25"/>
+      <c r="G262" s="25"/>
+      <c r="H262" s="26"/>
       <c r="I262" s="2"/>
       <c r="J262" s="2"/>
       <c r="K262" s="3"/>
@@ -7153,22 +7153,22 @@
       </c>
       <c r="B264" s="5"/>
       <c r="D264" t="s">
-        <v>379</v>
+        <v>393</v>
       </c>
       <c r="E264" s="7" t="s">
-        <v>380</v>
+        <v>394</v>
       </c>
       <c r="F264" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G264" s="6" t="s">
-        <v>381</v>
+        <v>395</v>
       </c>
       <c r="H264" s="6" t="s">
-        <v>382</v>
+        <v>396</v>
       </c>
       <c r="I264" s="6" t="s">
-        <v>383</v>
+        <v>397</v>
       </c>
       <c r="J264" s="15" t="s">
         <v>22</v>
@@ -7198,42 +7198,42 @@
       </c>
       <c r="B266" s="5"/>
       <c r="D266" t="s">
-        <v>493</v>
+        <v>398</v>
       </c>
       <c r="E266" s="7" t="s">
-        <v>384</v>
+        <v>399</v>
       </c>
       <c r="F266" s="6" t="s">
         <v>18</v>
       </c>
       <c r="G266" s="6" t="s">
-        <v>385</v>
+        <v>400</v>
       </c>
       <c r="H266" s="6" t="s">
-        <v>386</v>
+        <v>401</v>
       </c>
       <c r="I266" s="6" t="s">
-        <v>387</v>
+        <v>402</v>
       </c>
       <c r="J266" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K266" s="5"/>
       <c r="L266" s="5"/>
     </row>
     <row r="267" spans="1:12" ht="15.5" customHeight="1">
       <c r="A267" s="2" t="s">
-        <v>388</v>
+        <v>403</v>
       </c>
       <c r="B267" s="2"/>
       <c r="C267" s="2"/>
-      <c r="D267" s="26" t="s">
-        <v>389</v>
-      </c>
-      <c r="E267" s="27"/>
-      <c r="F267" s="27"/>
-      <c r="G267" s="27"/>
-      <c r="H267" s="28"/>
+      <c r="D267" s="24" t="s">
+        <v>404</v>
+      </c>
+      <c r="E267" s="25"/>
+      <c r="F267" s="25"/>
+      <c r="G267" s="25"/>
+      <c r="H267" s="26"/>
       <c r="I267" s="2"/>
       <c r="J267" s="2"/>
       <c r="K267" s="3"/>
@@ -7264,7 +7264,7 @@
       <c r="B269" s="1"/>
       <c r="C269" s="1"/>
       <c r="D269" s="21" t="s">
-        <v>390</v>
+        <v>405</v>
       </c>
       <c r="E269" s="15" t="s">
         <v>17</v>
@@ -7273,13 +7273,13 @@
         <v>18</v>
       </c>
       <c r="G269" s="16" t="s">
-        <v>391</v>
+        <v>406</v>
       </c>
       <c r="H269" s="16" t="s">
-        <v>392</v>
+        <v>407</v>
       </c>
       <c r="I269" s="16" t="s">
-        <v>393</v>
+        <v>408</v>
       </c>
       <c r="J269" s="15" t="s">
         <v>22</v>
@@ -7288,6 +7288,7 @@
       <c r="L269" s="1"/>
     </row>
     <row r="270" spans="1:12" ht="15.5" customHeight="1">
+      <c r="A270" s="1"/>
       <c r="B270" s="5"/>
       <c r="D270" s="1" t="s">
         <v>23</v>
@@ -7307,7 +7308,7 @@
       <c r="B271" s="1"/>
       <c r="C271" s="1"/>
       <c r="D271" s="21" t="s">
-        <v>394</v>
+        <v>409</v>
       </c>
       <c r="E271" s="15" t="s">
         <v>17</v>
@@ -7316,38 +7317,38 @@
         <v>18</v>
       </c>
       <c r="G271" s="16" t="s">
-        <v>395</v>
+        <v>410</v>
       </c>
       <c r="H271" s="16" t="s">
-        <v>396</v>
+        <v>411</v>
       </c>
       <c r="I271" s="16" t="s">
-        <v>397</v>
+        <v>412</v>
       </c>
       <c r="J271" s="15" t="s">
-        <v>398</v>
+        <v>413</v>
       </c>
       <c r="K271" s="1"/>
       <c r="L271" s="1"/>
     </row>
     <row r="272" spans="1:12" ht="15.5" customHeight="1">
       <c r="A272" s="2" t="s">
-        <v>399</v>
+        <v>414</v>
       </c>
       <c r="B272" s="2"/>
       <c r="C272" s="2"/>
-      <c r="D272" s="26" t="s">
-        <v>400</v>
-      </c>
-      <c r="E272" s="27"/>
-      <c r="F272" s="27"/>
-      <c r="G272" s="27"/>
-      <c r="H272" s="28"/>
+      <c r="D272" s="24" t="s">
+        <v>415</v>
+      </c>
+      <c r="E272" s="25"/>
+      <c r="F272" s="25"/>
+      <c r="G272" s="25"/>
+      <c r="H272" s="26"/>
       <c r="I272" s="2"/>
       <c r="J272" s="2"/>
       <c r="K272" s="3"/>
       <c r="L272" s="3" t="s">
-        <v>401</v>
+        <v>416</v>
       </c>
     </row>
     <row r="273" spans="1:12" ht="15.5" customHeight="1">
@@ -7412,17 +7413,17 @@
     </row>
     <row r="277" spans="1:12" ht="15.5" customHeight="1">
       <c r="A277" s="2" t="s">
-        <v>402</v>
+        <v>417</v>
       </c>
       <c r="B277" s="2"/>
       <c r="C277" s="2"/>
-      <c r="D277" s="26" t="s">
-        <v>403</v>
-      </c>
-      <c r="E277" s="27"/>
-      <c r="F277" s="27"/>
-      <c r="G277" s="27"/>
-      <c r="H277" s="28"/>
+      <c r="D277" s="24" t="s">
+        <v>418</v>
+      </c>
+      <c r="E277" s="25"/>
+      <c r="F277" s="25"/>
+      <c r="G277" s="25"/>
+      <c r="H277" s="26"/>
       <c r="I277" s="2"/>
       <c r="J277" s="2"/>
       <c r="K277" s="3"/>
@@ -7452,25 +7453,25 @@
       </c>
       <c r="B279" s="5"/>
       <c r="D279" t="s">
-        <v>404</v>
+        <v>419</v>
       </c>
       <c r="E279" s="7" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
       <c r="F279" s="6" t="s">
         <v>18</v>
       </c>
       <c r="G279" s="6" t="s">
-        <v>405</v>
+        <v>420</v>
       </c>
       <c r="H279" s="6" t="s">
-        <v>406</v>
+        <v>421</v>
       </c>
       <c r="I279" s="6" t="s">
-        <v>407</v>
+        <v>422</v>
       </c>
       <c r="J279" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K279" s="5"/>
       <c r="L279" s="5"/>
@@ -7507,17 +7508,17 @@
     </row>
     <row r="282" spans="1:12" ht="15.5" customHeight="1">
       <c r="A282" s="2" t="s">
-        <v>408</v>
+        <v>423</v>
       </c>
       <c r="B282" s="2"/>
       <c r="C282" s="2"/>
-      <c r="D282" s="26" t="s">
-        <v>409</v>
-      </c>
-      <c r="E282" s="27"/>
-      <c r="F282" s="27"/>
-      <c r="G282" s="27"/>
-      <c r="H282" s="28"/>
+      <c r="D282" s="24" t="s">
+        <v>424</v>
+      </c>
+      <c r="E282" s="25"/>
+      <c r="F282" s="25"/>
+      <c r="G282" s="25"/>
+      <c r="H282" s="26"/>
       <c r="I282" s="2"/>
       <c r="J282" s="2"/>
       <c r="K282" s="3"/>
@@ -7547,25 +7548,25 @@
       </c>
       <c r="B284" s="5"/>
       <c r="D284" t="s">
-        <v>410</v>
+        <v>425</v>
       </c>
       <c r="E284" s="7" t="s">
-        <v>411</v>
+        <v>426</v>
       </c>
       <c r="F284" s="6" t="s">
         <v>18</v>
       </c>
       <c r="G284" s="6" t="s">
-        <v>412</v>
+        <v>427</v>
       </c>
       <c r="H284" s="6" t="s">
-        <v>413</v>
+        <v>428</v>
       </c>
       <c r="I284" s="6" t="s">
-        <v>414</v>
+        <v>429</v>
       </c>
       <c r="J284" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K284" s="5"/>
       <c r="L284" s="5"/>
@@ -7592,42 +7593,42 @@
       </c>
       <c r="B286" s="5"/>
       <c r="D286" t="s">
-        <v>415</v>
+        <v>430</v>
       </c>
       <c r="E286" s="7" t="s">
-        <v>416</v>
+        <v>431</v>
       </c>
       <c r="F286" s="6" t="s">
         <v>18</v>
       </c>
       <c r="G286" s="6" t="s">
-        <v>417</v>
+        <v>432</v>
       </c>
       <c r="H286" s="6" t="s">
-        <v>418</v>
+        <v>433</v>
       </c>
       <c r="I286" s="6" t="s">
-        <v>419</v>
+        <v>434</v>
       </c>
       <c r="J286" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K286" s="5"/>
       <c r="L286" s="5"/>
     </row>
     <row r="287" spans="1:12" ht="15.5" customHeight="1">
       <c r="A287" s="2" t="s">
-        <v>420</v>
+        <v>435</v>
       </c>
       <c r="B287" s="2"/>
       <c r="C287" s="2"/>
-      <c r="D287" s="26" t="s">
-        <v>421</v>
-      </c>
-      <c r="E287" s="27"/>
-      <c r="F287" s="27"/>
-      <c r="G287" s="27"/>
-      <c r="H287" s="28"/>
+      <c r="D287" s="24" t="s">
+        <v>436</v>
+      </c>
+      <c r="E287" s="25"/>
+      <c r="F287" s="25"/>
+      <c r="G287" s="25"/>
+      <c r="H287" s="26"/>
       <c r="I287" s="2"/>
       <c r="J287" s="2"/>
       <c r="K287" s="3"/>
@@ -7657,25 +7658,25 @@
       </c>
       <c r="B289" s="5"/>
       <c r="D289" t="s">
-        <v>494</v>
+        <v>437</v>
       </c>
       <c r="E289" s="7" t="s">
-        <v>267</v>
+        <v>278</v>
       </c>
       <c r="F289" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G289" s="6" t="s">
-        <v>422</v>
+        <v>438</v>
       </c>
       <c r="H289" s="6" t="s">
-        <v>423</v>
+        <v>439</v>
       </c>
       <c r="I289" s="6" t="s">
-        <v>424</v>
+        <v>440</v>
       </c>
       <c r="J289" s="7" t="s">
-        <v>376</v>
+        <v>390</v>
       </c>
       <c r="K289" s="5"/>
       <c r="L289" s="5"/>
@@ -7712,17 +7713,17 @@
     </row>
     <row r="292" spans="1:12" ht="15.5" customHeight="1">
       <c r="A292" s="2" t="s">
-        <v>425</v>
+        <v>441</v>
       </c>
       <c r="B292" s="2"/>
       <c r="C292" s="2"/>
-      <c r="D292" s="26" t="s">
-        <v>426</v>
-      </c>
-      <c r="E292" s="27"/>
-      <c r="F292" s="27"/>
-      <c r="G292" s="27"/>
-      <c r="H292" s="28"/>
+      <c r="D292" s="24" t="s">
+        <v>442</v>
+      </c>
+      <c r="E292" s="25"/>
+      <c r="F292" s="25"/>
+      <c r="G292" s="25"/>
+      <c r="H292" s="26"/>
       <c r="I292" s="2"/>
       <c r="J292" s="2"/>
       <c r="K292" s="3"/>
@@ -7752,25 +7753,25 @@
       </c>
       <c r="B294" s="5"/>
       <c r="D294" t="s">
-        <v>495</v>
+        <v>443</v>
       </c>
       <c r="E294" s="7" t="s">
-        <v>427</v>
+        <v>444</v>
       </c>
       <c r="F294" s="6" t="s">
         <v>18</v>
       </c>
       <c r="G294" s="6" t="s">
-        <v>428</v>
+        <v>445</v>
       </c>
       <c r="H294" s="6" t="s">
-        <v>429</v>
+        <v>446</v>
       </c>
       <c r="I294" s="6" t="s">
-        <v>430</v>
+        <v>447</v>
       </c>
       <c r="J294" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K294" s="5"/>
       <c r="L294" s="5"/>
@@ -7807,17 +7808,17 @@
     </row>
     <row r="297" spans="1:12" ht="15.5" customHeight="1">
       <c r="A297" s="2" t="s">
-        <v>431</v>
+        <v>448</v>
       </c>
       <c r="B297" s="2"/>
       <c r="C297" s="2"/>
-      <c r="D297" s="26" t="s">
-        <v>432</v>
-      </c>
-      <c r="E297" s="27"/>
-      <c r="F297" s="27"/>
-      <c r="G297" s="27"/>
-      <c r="H297" s="28"/>
+      <c r="D297" s="24" t="s">
+        <v>449</v>
+      </c>
+      <c r="E297" s="25"/>
+      <c r="F297" s="25"/>
+      <c r="G297" s="25"/>
+      <c r="H297" s="26"/>
       <c r="I297" s="2"/>
       <c r="J297" s="2"/>
       <c r="K297" s="3"/>
@@ -7847,25 +7848,25 @@
       </c>
       <c r="B299" s="5"/>
       <c r="D299" t="s">
-        <v>496</v>
+        <v>450</v>
       </c>
       <c r="E299" s="7" t="s">
-        <v>433</v>
+        <v>451</v>
       </c>
       <c r="F299" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G299" s="6" t="s">
-        <v>434</v>
+        <v>452</v>
       </c>
       <c r="H299" s="6" t="s">
-        <v>435</v>
+        <v>453</v>
       </c>
       <c r="I299" s="6" t="s">
-        <v>436</v>
+        <v>454</v>
       </c>
       <c r="J299" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="K299" s="5"/>
       <c r="L299" s="5"/>
@@ -7902,17 +7903,17 @@
     </row>
     <row r="302" spans="1:12" ht="15.5" customHeight="1">
       <c r="A302" s="2" t="s">
-        <v>437</v>
+        <v>455</v>
       </c>
       <c r="B302" s="2"/>
       <c r="C302" s="2"/>
-      <c r="D302" s="26" t="s">
-        <v>438</v>
-      </c>
-      <c r="E302" s="27"/>
-      <c r="F302" s="27"/>
-      <c r="G302" s="27"/>
-      <c r="H302" s="28"/>
+      <c r="D302" s="24" t="s">
+        <v>456</v>
+      </c>
+      <c r="E302" s="25"/>
+      <c r="F302" s="25"/>
+      <c r="G302" s="25"/>
+      <c r="H302" s="26"/>
       <c r="I302" s="2"/>
       <c r="J302" s="2"/>
       <c r="K302" s="3"/>
@@ -7942,25 +7943,25 @@
       </c>
       <c r="B304" s="5"/>
       <c r="D304" s="21" t="s">
-        <v>439</v>
+        <v>457</v>
       </c>
       <c r="E304" s="15" t="s">
         <v>17</v>
       </c>
       <c r="F304" s="16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G304" s="16" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H304" s="16" t="s">
-        <v>441</v>
+        <v>459</v>
       </c>
       <c r="I304" s="16" t="s">
-        <v>442</v>
+        <v>460</v>
       </c>
       <c r="J304" s="15" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="K304" s="5"/>
       <c r="L304" s="5"/>
@@ -7997,17 +7998,17 @@
     </row>
     <row r="307" spans="1:12" ht="15.5" customHeight="1">
       <c r="A307" s="2" t="s">
-        <v>443</v>
+        <v>461</v>
       </c>
       <c r="B307" s="2"/>
       <c r="C307" s="2"/>
-      <c r="D307" s="26" t="s">
-        <v>444</v>
-      </c>
-      <c r="E307" s="27"/>
-      <c r="F307" s="27"/>
-      <c r="G307" s="27"/>
-      <c r="H307" s="28"/>
+      <c r="D307" s="24" t="s">
+        <v>462</v>
+      </c>
+      <c r="E307" s="25"/>
+      <c r="F307" s="25"/>
+      <c r="G307" s="25"/>
+      <c r="H307" s="26"/>
       <c r="I307" s="2"/>
       <c r="J307" s="2"/>
       <c r="K307" s="3"/>
@@ -8037,25 +8038,25 @@
       </c>
       <c r="B309" s="5"/>
       <c r="D309" t="s">
-        <v>445</v>
+        <v>463</v>
       </c>
       <c r="E309" s="7" t="s">
-        <v>446</v>
+        <v>464</v>
       </c>
       <c r="F309" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G309" s="6" t="s">
-        <v>447</v>
+        <v>465</v>
       </c>
       <c r="H309" s="6" t="s">
-        <v>448</v>
+        <v>466</v>
       </c>
       <c r="I309" s="6" t="s">
-        <v>449</v>
+        <v>467</v>
       </c>
       <c r="J309" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="K309" s="5"/>
       <c r="L309" s="5"/>
@@ -8092,17 +8093,17 @@
     </row>
     <row r="312" spans="1:12" ht="15.5" customHeight="1">
       <c r="A312" s="2" t="s">
-        <v>450</v>
+        <v>468</v>
       </c>
       <c r="B312" s="2"/>
       <c r="C312" s="2"/>
-      <c r="D312" s="26" t="s">
-        <v>451</v>
-      </c>
-      <c r="E312" s="27"/>
-      <c r="F312" s="27"/>
-      <c r="G312" s="27"/>
-      <c r="H312" s="28"/>
+      <c r="D312" s="24" t="s">
+        <v>469</v>
+      </c>
+      <c r="E312" s="25"/>
+      <c r="F312" s="25"/>
+      <c r="G312" s="25"/>
+      <c r="H312" s="26"/>
       <c r="I312" s="2"/>
       <c r="J312" s="2"/>
       <c r="K312" s="3"/>
@@ -8132,25 +8133,25 @@
       </c>
       <c r="B314" s="5"/>
       <c r="D314" s="21" t="s">
-        <v>452</v>
+        <v>470</v>
       </c>
       <c r="E314" s="15" t="s">
         <v>17</v>
       </c>
       <c r="F314" s="16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G314" s="16" t="s">
-        <v>453</v>
+        <v>471</v>
       </c>
       <c r="H314" s="16" t="s">
-        <v>454</v>
+        <v>472</v>
       </c>
       <c r="I314" s="16" t="s">
-        <v>455</v>
+        <v>473</v>
       </c>
       <c r="J314" s="15" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="K314" s="5"/>
       <c r="L314" s="5"/>
@@ -8177,42 +8178,42 @@
       </c>
       <c r="B316" s="5"/>
       <c r="D316" t="s">
-        <v>456</v>
+        <v>474</v>
       </c>
       <c r="E316" s="7" t="s">
-        <v>457</v>
+        <v>475</v>
       </c>
       <c r="F316" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G316" s="6" t="s">
-        <v>458</v>
+        <v>476</v>
       </c>
       <c r="H316" s="6" t="s">
-        <v>459</v>
+        <v>477</v>
       </c>
       <c r="I316" s="6" t="s">
-        <v>460</v>
+        <v>478</v>
       </c>
       <c r="J316" s="7" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="K316" s="5"/>
       <c r="L316" s="5"/>
     </row>
     <row r="317" spans="1:12" ht="15.5" customHeight="1">
       <c r="A317" s="2" t="s">
-        <v>461</v>
+        <v>479</v>
       </c>
       <c r="B317" s="2"/>
       <c r="C317" s="2"/>
-      <c r="D317" s="26" t="s">
-        <v>462</v>
-      </c>
-      <c r="E317" s="27"/>
-      <c r="F317" s="27"/>
-      <c r="G317" s="27"/>
-      <c r="H317" s="28"/>
+      <c r="D317" s="24" t="s">
+        <v>480</v>
+      </c>
+      <c r="E317" s="25"/>
+      <c r="F317" s="25"/>
+      <c r="G317" s="25"/>
+      <c r="H317" s="26"/>
       <c r="I317" s="2"/>
       <c r="J317" s="2"/>
       <c r="K317" s="3"/>
@@ -8242,7 +8243,7 @@
       </c>
       <c r="B319" s="5"/>
       <c r="D319" s="21" t="s">
-        <v>463</v>
+        <v>481</v>
       </c>
       <c r="E319" s="15" t="s">
         <v>17</v>
@@ -8251,16 +8252,16 @@
         <v>18</v>
       </c>
       <c r="G319" s="16" t="s">
-        <v>464</v>
+        <v>482</v>
       </c>
       <c r="H319" s="16" t="s">
-        <v>465</v>
+        <v>483</v>
       </c>
       <c r="I319" s="16" t="s">
-        <v>466</v>
+        <v>484</v>
       </c>
       <c r="J319" s="15" t="s">
-        <v>467</v>
+        <v>485</v>
       </c>
       <c r="K319" s="5"/>
       <c r="L319" s="5"/>
@@ -8287,42 +8288,42 @@
       </c>
       <c r="B321" s="5"/>
       <c r="D321" s="21" t="s">
-        <v>468</v>
+        <v>486</v>
       </c>
       <c r="E321" s="15" t="s">
         <v>17</v>
       </c>
       <c r="F321" s="16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G321" s="16" t="s">
-        <v>469</v>
+        <v>487</v>
       </c>
       <c r="H321" s="16" t="s">
-        <v>470</v>
+        <v>488</v>
       </c>
       <c r="I321" s="16" t="s">
-        <v>471</v>
+        <v>489</v>
       </c>
       <c r="J321" s="15" t="s">
-        <v>467</v>
+        <v>485</v>
       </c>
       <c r="K321" s="5"/>
       <c r="L321" s="5"/>
     </row>
     <row r="322" spans="1:12" ht="15.5" customHeight="1">
       <c r="A322" s="2" t="s">
-        <v>472</v>
+        <v>490</v>
       </c>
       <c r="B322" s="2"/>
       <c r="C322" s="2"/>
-      <c r="D322" s="26" t="s">
-        <v>473</v>
-      </c>
-      <c r="E322" s="27"/>
-      <c r="F322" s="27"/>
-      <c r="G322" s="27"/>
-      <c r="H322" s="28"/>
+      <c r="D322" s="24" t="s">
+        <v>491</v>
+      </c>
+      <c r="E322" s="25"/>
+      <c r="F322" s="25"/>
+      <c r="G322" s="25"/>
+      <c r="H322" s="26"/>
       <c r="I322" s="2"/>
       <c r="J322" s="2"/>
       <c r="K322" s="3"/>
@@ -8352,25 +8353,25 @@
       </c>
       <c r="B324" s="5"/>
       <c r="D324" t="s">
-        <v>497</v>
+        <v>492</v>
       </c>
       <c r="E324" s="7" t="s">
-        <v>474</v>
+        <v>493</v>
       </c>
       <c r="F324" s="6" t="s">
         <v>18</v>
       </c>
       <c r="G324" s="6" t="s">
-        <v>475</v>
+        <v>494</v>
       </c>
       <c r="H324" s="6" t="s">
-        <v>476</v>
+        <v>495</v>
       </c>
       <c r="I324" s="6" t="s">
-        <v>477</v>
+        <v>496</v>
       </c>
       <c r="J324" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K324" s="5"/>
       <c r="L324" s="5"/>
@@ -8408,25 +8409,64 @@
       <c r="L326" s="5"/>
     </row>
     <row r="328" spans="1:12">
-      <c r="H328" s="24" t="s">
-        <v>478</v>
-      </c>
-      <c r="I328" s="25"/>
+      <c r="H328" s="27" t="s">
+        <v>497</v>
+      </c>
+      <c r="I328" s="28"/>
     </row>
     <row r="330" spans="1:12">
-      <c r="H330" s="24" t="s">
-        <v>479</v>
-      </c>
-      <c r="I330" s="25"/>
+      <c r="H330" s="27" t="s">
+        <v>498</v>
+      </c>
+      <c r="I330" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="67">
-    <mergeCell ref="D182:H182"/>
-    <mergeCell ref="D172:H172"/>
-    <mergeCell ref="D262:H262"/>
-    <mergeCell ref="D187:H187"/>
-    <mergeCell ref="D247:H247"/>
+    <mergeCell ref="H328:I328"/>
+    <mergeCell ref="D222:H222"/>
+    <mergeCell ref="D322:H322"/>
+    <mergeCell ref="D82:H82"/>
+    <mergeCell ref="D67:H67"/>
+    <mergeCell ref="D142:H142"/>
+    <mergeCell ref="D207:H207"/>
+    <mergeCell ref="D132:H132"/>
     <mergeCell ref="D252:H252"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="D152:H152"/>
+    <mergeCell ref="D192:H192"/>
+    <mergeCell ref="D117:H117"/>
+    <mergeCell ref="D232:H232"/>
+    <mergeCell ref="D157:H157"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D177:H177"/>
+    <mergeCell ref="D122:H122"/>
+    <mergeCell ref="D212:H212"/>
+    <mergeCell ref="D102:H102"/>
+    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D317:H317"/>
+    <mergeCell ref="D137:H137"/>
+    <mergeCell ref="D62:H62"/>
+    <mergeCell ref="D202:H202"/>
+    <mergeCell ref="D307:H307"/>
+    <mergeCell ref="D167:H167"/>
+    <mergeCell ref="D127:H127"/>
+    <mergeCell ref="D92:H92"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="D297:H297"/>
+    <mergeCell ref="D27:H27"/>
+    <mergeCell ref="D287:H287"/>
+    <mergeCell ref="D107:H107"/>
+    <mergeCell ref="D32:H32"/>
+    <mergeCell ref="D277:H277"/>
+    <mergeCell ref="D272:H272"/>
+    <mergeCell ref="D97:H97"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D197:H197"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D162:H162"/>
+    <mergeCell ref="D47:H47"/>
+    <mergeCell ref="D87:H87"/>
+    <mergeCell ref="D227:H227"/>
     <mergeCell ref="H330:I330"/>
     <mergeCell ref="D237:H237"/>
     <mergeCell ref="D217:H217"/>
@@ -8443,51 +8483,12 @@
     <mergeCell ref="D292:H292"/>
     <mergeCell ref="D72:H72"/>
     <mergeCell ref="D112:H112"/>
-    <mergeCell ref="D162:H162"/>
-    <mergeCell ref="D47:H47"/>
-    <mergeCell ref="D87:H87"/>
-    <mergeCell ref="D67:H67"/>
-    <mergeCell ref="D132:H132"/>
-    <mergeCell ref="D92:H92"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D27:H27"/>
-    <mergeCell ref="D107:H107"/>
-    <mergeCell ref="D32:H32"/>
-    <mergeCell ref="D97:H97"/>
-    <mergeCell ref="D17:H17"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D12:H12"/>
-    <mergeCell ref="D152:H152"/>
-    <mergeCell ref="D192:H192"/>
-    <mergeCell ref="D117:H117"/>
-    <mergeCell ref="D232:H232"/>
-    <mergeCell ref="D157:H157"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D177:H177"/>
-    <mergeCell ref="D122:H122"/>
-    <mergeCell ref="D212:H212"/>
-    <mergeCell ref="D102:H102"/>
-    <mergeCell ref="D37:H37"/>
-    <mergeCell ref="D137:H137"/>
-    <mergeCell ref="D62:H62"/>
-    <mergeCell ref="D167:H167"/>
-    <mergeCell ref="D127:H127"/>
-    <mergeCell ref="H328:I328"/>
-    <mergeCell ref="D222:H222"/>
-    <mergeCell ref="D322:H322"/>
-    <mergeCell ref="D82:H82"/>
-    <mergeCell ref="D142:H142"/>
-    <mergeCell ref="D207:H207"/>
-    <mergeCell ref="D317:H317"/>
-    <mergeCell ref="D202:H202"/>
-    <mergeCell ref="D307:H307"/>
-    <mergeCell ref="D297:H297"/>
-    <mergeCell ref="D287:H287"/>
-    <mergeCell ref="D277:H277"/>
-    <mergeCell ref="D272:H272"/>
-    <mergeCell ref="D197:H197"/>
-    <mergeCell ref="D227:H227"/>
     <mergeCell ref="D302:H302"/>
+    <mergeCell ref="D182:H182"/>
+    <mergeCell ref="D172:H172"/>
+    <mergeCell ref="D262:H262"/>
+    <mergeCell ref="D187:H187"/>
+    <mergeCell ref="D247:H247"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="B4 B6 B9 B11 B14 B16 B19 B21 B24 B26 B29 B31 B34 B36 B39 B41 B44 B46 B49 B51 B54 B56 B59 B61 B64 B66 B69 B71 B74 B76 B79 B81 B84 B86 B89 B91 B94 B96 B99 B101 B104 B106 B109 B111 B114 B116 B119 B121 B124 B126 B129 B131 B134 B136 B139 B141 B144 B146 B149 B151 B154 B156 B159 B161 B164 B166 B169 B171 B174 B176 B179 B181 B184 B186 B189 B191 B194 B196 B199 B201 B204 B206 B209 B211 B214 B216 B219 B221 B224 B226 B229 B231 B234 B236 B239 B241 B244 B246 B249 B251 B254 B256 B259 B261 B264 B266 B270 B274 B276 B279 B281 B284 B286 B289 B291 B294 B296 B299 B301 B304 B306 B309 B311 B314 B316 B319 B321 B324 B326" xr:uid="{00000000-0002-0000-0000-000000000000}">

</xml_diff>